<commit_message>
Quality and assumption audit: access guard, approval and step gates, state integrity, responsive fixes
Administration route guard; approval handlers re-check authority; forward jumps need valid steps; submits require eligibility; line must belong to the identified customer; failed config load fails approvals closed; held plan changes apply on approval; role switch resolves identity first; draft writes go through the entity store; Drawer and form grids fit small screens; tests for each.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
+++ b/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB36E25-6106-5345-BE99-D9E23F697C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A34264-D39C-6B46-8D33-0A14DF4D9A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1000" windowWidth="34560" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Identity scan, plan-step and sign-in polish: scanner wording, route scroll, HRN demo scan, single Special Discount, password toggle
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
+++ b/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
@@ -19,12 +19,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customers'!$A$1:$AH$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customers'!$A$1:$AH$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scenario Coverage'!$A$1:$D$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Eligibility Coverage'!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Retired &amp; MADA QIDs'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Eligibility Coverage1'!$A$1:$H$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Seeded Records'!$A$1:$D$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Seeded Records'!$A$1:$D$131</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Roles &amp; Login'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Journey Access by Role'!$A$1:$N$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Open Questions'!$A$1:$E$11</definedName>
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>68 test customers, ALL loaded in the running app: 10 original demo records and 58 added on 02/10/2026 by this script's --seed step (see 'Seeded Records').</t>
+          <t>69 test customers, ALL loaded in the running app: 10 original demo records and 59 added on 02/10/2026 by this script's --seed step (see 'Seeded Records').</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH69"/>
+  <dimension ref="A1:AH70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.15" customWidth="1" min="1" max="1"/>
@@ -7276,54 +7276,54 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>TC-040</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>CUST-1003</t>
-        </is>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>In app - original</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>5 Existing - no mobile line</t>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>NAS-7006</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>In app - added 02/10/2026</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>4 New customer / MNP</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>Fatima Saud Hamad Al-Kuwari</t>
+          <t>Farhan Aslam Javed Chaudhry</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr">
         <is>
-          <t>Fatima</t>
+          <t>Farhan</t>
         </is>
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>Saud Hamad</t>
+          <t>Aslam Javed</t>
         </is>
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
-          <t>Al-Kuwari</t>
+          <t>Chaudhry</t>
         </is>
       </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Pakistani</t>
         </is>
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K41" s="13" t="inlineStr">
@@ -7333,53 +7333,45 @@
       </c>
       <c r="L41" s="13" t="inlineStr">
         <is>
-          <t>27798765432</t>
+          <t>29303051200106</t>
         </is>
       </c>
       <c r="M41" s="13" t="inlineStr">
         <is>
-          <t>30/11/2029</t>
+          <t>31/10/2030</t>
         </is>
       </c>
       <c r="N41" s="13" t="inlineStr">
         <is>
-          <t>05/11/1978</t>
+          <t>05/03/1993</t>
         </is>
       </c>
       <c r="O41" s="13" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="P41" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q41" s="13" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Not a customer</t>
         </is>
       </c>
       <c r="R41" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
-        </is>
-      </c>
-      <c r="S41" s="13" t="inlineStr">
-        <is>
-          <t>+97455512003</t>
-        </is>
-      </c>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="S41" s="13" t="inlineStr"/>
       <c r="T41" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="U41" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V41" s="13" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="U41" s="13" t="inlineStr"/>
+      <c r="V41" s="13" t="inlineStr"/>
       <c r="W41" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X41" s="13" t="n">
         <v>0</v>
@@ -7391,33 +7383,33 @@
       </c>
       <c r="Z41" s="13" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>HRN</t>
         </is>
       </c>
       <c r="AA41" s="13" t="inlineStr"/>
       <c r="AB41" s="13" t="inlineStr">
         <is>
-          <t>Loyalty (existing customer)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="AC41" s="13" t="inlineStr">
         <is>
-          <t>FNP-12001 (Ooredoo donor validation); POUT-17003 FNP conditional accept</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD41" s="13" t="inlineStr">
         <is>
-          <t>Qatari with a GigaHome fixed-line account only (0 mobile lines). Existing customer, two draft orders, FNP port-in in progress.</t>
+          <t>NEW HRN customer (NAS only, Pakistani). The New Customer journey's demo scan always returns this person, so a demo New Customer is HRN-category.</t>
         </is>
       </c>
       <c r="AE41" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid for an existing fixed-line customer; Fixed Line; FNP</t>
+          <t>New Postpaid; New Prepaid</t>
         </is>
       </c>
       <c r="AF41" s="13" t="inlineStr">
         <is>
-          <t>Identifies as EXISTING customer even with 0 active lines. All eligibility checks pass.</t>
+          <t>Resolves via NAS, no customerId. HRN: QAR 100 advance, QAR 50 default credit limit, no limit choice (hrnConfiguration). The scanned card, the number read and the MOI result are this one person, so ID reconciliation passes.</t>
         </is>
       </c>
       <c r="AG41" s="13" t="inlineStr">
@@ -7427,7 +7419,7 @@
       </c>
       <c r="AH41" s="13" t="inlineStr">
         <is>
-          <t>Original demo data: customers.json, identity-documents.json</t>
+          <t>Synthetic record.</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7431,7 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>CUST-1004</t>
+          <t>CUST-1003</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
@@ -7449,27 +7441,27 @@
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>6 Eligibility gates</t>
+          <t>5 Existing - no mobile line</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>Mohammed Rashid Khalid Al-Emadi</t>
+          <t>Fatima Saud Hamad Al-Kuwari</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>Mohammed</t>
+          <t>Fatima</t>
         </is>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Rashid Khalid</t>
+          <t>Saud Hamad</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>Al-Emadi</t>
+          <t>Al-Kuwari</t>
         </is>
       </c>
       <c r="I42" s="13" t="inlineStr">
@@ -7489,7 +7481,7 @@
       </c>
       <c r="L42" s="13" t="inlineStr">
         <is>
-          <t>29011122233</t>
+          <t>27798765432</t>
         </is>
       </c>
       <c r="M42" s="13" t="inlineStr">
@@ -7499,15 +7491,15 @@
       </c>
       <c r="N42" s="13" t="inlineStr">
         <is>
-          <t>30/01/1995</t>
+          <t>05/11/1978</t>
         </is>
       </c>
       <c r="O42" s="13" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="P42" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q42" s="13" t="inlineStr">
@@ -7517,16 +7509,16 @@
       </c>
       <c r="R42" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
-          <t>+97455512004</t>
+          <t>+97455512003</t>
         </is>
       </c>
       <c r="T42" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U42" s="13" t="n">
         <v>0</v>
@@ -7538,11 +7530,11 @@
         <v>1</v>
       </c>
       <c r="X42" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y42" s="13" t="inlineStr">
         <is>
-          <t>collections</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z42" s="13" t="inlineStr">
@@ -7553,27 +7545,27 @@
       <c r="AA42" s="13" t="inlineStr"/>
       <c r="AB42" s="13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Loyalty (existing customer)</t>
         </is>
       </c>
       <c r="AC42" s="13" t="inlineStr">
         <is>
-          <t>MNP-11002 donor conditional-accept (billed due over QAR 100)</t>
+          <t>FNP-12001 (Ooredoo donor validation); POUT-17003 FNP conditional accept</t>
         </is>
       </c>
       <c r="AD42" s="13" t="inlineStr">
         <is>
-          <t>Qatari, collections-blacklisted (outstanding dues above threshold). Postpaid blocked, prepaid still offered.</t>
+          <t>Qatari with a GigaHome fixed-line account only (0 mobile lines). Existing customer, two draft orders, FNP port-in in progress.</t>
         </is>
       </c>
       <c r="AE42" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid (soft-stop); New Prepaid; MNP</t>
+          <t>New Postpaid for an existing fixed-line customer; Fixed Line; FNP</t>
         </is>
       </c>
       <c r="AF42" s="13" t="inlineStr">
         <is>
-          <t>Collections Check = soft-stop: 'Postpaid cannot be issued. Prepaid is available on this QID.' (BR-113: blacklist only, never the balance).</t>
+          <t>Identifies as EXISTING customer even with 0 active lines. All eligibility checks pass.</t>
         </is>
       </c>
       <c r="AG42" s="13" t="inlineStr">
@@ -7595,7 +7587,7 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>CUST-1006</t>
+          <t>CUST-1004</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
@@ -7610,60 +7602,60 @@
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>Sophie Marie Laurent</t>
+          <t>Mohammed Rashid Khalid Al-Emadi</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
         <is>
-          <t>Sophie</t>
+          <t>Mohammed</t>
         </is>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Marie</t>
+          <t>Rashid Khalid</t>
         </is>
       </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
-          <t>Laurent</t>
+          <t>Al-Emadi</t>
         </is>
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>French</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>Expat</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>Diplomatic ID</t>
+          <t>QID</t>
         </is>
       </c>
       <c r="L43" s="13" t="inlineStr">
         <is>
-          <t>DIP-QA-004521</t>
+          <t>29011122233</t>
         </is>
       </c>
       <c r="M43" s="13" t="inlineStr">
         <is>
-          <t>31/08/2025</t>
+          <t>30/11/2029</t>
         </is>
       </c>
       <c r="N43" s="13" t="inlineStr">
         <is>
-          <t>02/04/1979</t>
+          <t>30/01/1995</t>
         </is>
       </c>
       <c r="O43" s="13" t="n">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="P43" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q43" s="13" t="inlineStr">
@@ -7678,11 +7670,11 @@
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
-          <t>+97455512007</t>
+          <t>+97455512004</t>
         </is>
       </c>
       <c r="T43" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U43" s="13" t="n">
         <v>0</v>
@@ -7691,14 +7683,14 @@
         <v>0</v>
       </c>
       <c r="W43" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X43" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y43" s="13" t="inlineStr">
         <is>
-          <t>security</t>
+          <t>collections</t>
         </is>
       </c>
       <c r="Z43" s="13" t="inlineStr">
@@ -7714,22 +7706,22 @@
       </c>
       <c r="AC43" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MNP-11002 donor conditional-accept (billed due over QAR 100)</t>
         </is>
       </c>
       <c r="AD43" s="13" t="inlineStr">
         <is>
-          <t>French diplomat, Diplomatic ID EXPIRED 31/08/2025, security-blacklisted.</t>
+          <t>Qatari, collections-blacklisted (outstanding dues above threshold). Postpaid blocked, prepaid still offered.</t>
         </is>
       </c>
       <c r="AE43" s="13" t="inlineStr">
         <is>
-          <t>Any new connection</t>
+          <t>New Postpaid (soft-stop); New Prepaid; MNP</t>
         </is>
       </c>
       <c r="AF43" s="13" t="inlineStr">
         <is>
-          <t>ID Validity hard-stop (expired) AND Security Check hard-stop. No agent override.</t>
+          <t>Collections Check = soft-stop: 'Postpaid cannot be issued. Prepaid is available on this QID.' (BR-113: blacklist only, never the balance).</t>
         </is>
       </c>
       <c r="AG43" s="13" t="inlineStr">
@@ -7751,7 +7743,7 @@
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>CUST-1007</t>
+          <t>CUST-1006</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
@@ -7766,27 +7758,27 @@
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>Henrik Lars Lindqvist</t>
+          <t>Sophie Marie Laurent</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Sophie</t>
         </is>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>Lars</t>
+          <t>Marie</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>Lindqvist</t>
+          <t>Laurent</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Swedish</t>
+          <t>French</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
@@ -7801,25 +7793,25 @@
       </c>
       <c r="L44" s="13" t="inlineStr">
         <is>
-          <t>DIP-QA-004977</t>
+          <t>DIP-QA-004521</t>
         </is>
       </c>
       <c r="M44" s="13" t="inlineStr">
         <is>
-          <t>30/04/2030</t>
+          <t>31/08/2025</t>
         </is>
       </c>
       <c r="N44" s="13" t="inlineStr">
         <is>
-          <t>11/02/1981</t>
+          <t>02/04/1979</t>
         </is>
       </c>
       <c r="O44" s="13" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P44" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q44" s="13" t="inlineStr">
@@ -7834,7 +7826,7 @@
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
-          <t>+97455512008</t>
+          <t>+97455512007</t>
         </is>
       </c>
       <c r="T44" s="13" t="n">
@@ -7854,7 +7846,7 @@
       </c>
       <c r="Y44" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>security</t>
         </is>
       </c>
       <c r="Z44" s="13" t="inlineStr">
@@ -7875,17 +7867,17 @@
       </c>
       <c r="AD44" s="13" t="inlineStr">
         <is>
-          <t>Swedish resident whose customers.json idType is QID but whose only document is a valid Diplomatic ID (to 30/04/2030).</t>
+          <t>French diplomat, Diplomatic ID EXPIRED 31/08/2025, security-blacklisted.</t>
         </is>
       </c>
       <c r="AE44" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid</t>
+          <t>Any new connection</t>
         </is>
       </c>
       <c r="AF44" s="13" t="inlineStr">
         <is>
-          <t>Document type governs: Diplomatic ID is exception-routed to Back Office Fulfilment approval.</t>
+          <t>ID Validity hard-stop (expired) AND Security Check hard-stop. No agent override.</t>
         </is>
       </c>
       <c r="AG44" s="13" t="inlineStr">
@@ -7900,78 +7892,78 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>TC-044</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>CUST-3041</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="inlineStr">
-        <is>
-          <t>In app - added 02/10/2026</t>
-        </is>
-      </c>
-      <c r="D45" s="14" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>CUST-1007</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>In app - original</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>6 Eligibility gates</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>Omar Samer Khalil Al-Hamwi</t>
+          <t>Henrik Lars Lindqvist</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>Henrik</t>
         </is>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Samer Khalil</t>
+          <t>Lars</t>
         </is>
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Al-Hamwi</t>
+          <t>Lindqvist</t>
         </is>
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>Syrian</t>
+          <t>Swedish</t>
         </is>
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>Expat (QID)</t>
+          <t>Expat</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>QID</t>
+          <t>Diplomatic ID</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
         <is>
-          <t>28808076000041</t>
+          <t>DIP-QA-004977</t>
         </is>
       </c>
       <c r="M45" s="13" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>30/04/2030</t>
         </is>
       </c>
       <c r="N45" s="13" t="inlineStr">
         <is>
-          <t>30/08/1988</t>
+          <t>11/02/1981</t>
         </is>
       </c>
       <c r="O45" s="13" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="P45" s="13" t="inlineStr">
         <is>
@@ -7985,19 +7977,19 @@
       </c>
       <c r="R45" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
-          <t>+97455513027</t>
+          <t>+97455512008</t>
         </is>
       </c>
       <c r="T45" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U45" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V45" s="13" t="n">
         <v>0</v>
@@ -8031,17 +8023,17 @@
       </c>
       <c r="AD45" s="13" t="inlineStr">
         <is>
-          <t>Expat whose QID EXPIRED on 31/12/2025.</t>
+          <t>Swedish resident whose customers.json idType is QID but whose only document is a valid Diplomatic ID (to 30/04/2030).</t>
         </is>
       </c>
       <c r="AE45" s="13" t="inlineStr">
         <is>
-          <t>Any new connection</t>
+          <t>New Postpaid</t>
         </is>
       </c>
       <c r="AF45" s="13" t="inlineStr">
         <is>
-          <t>ID Validity hard-stop: 'This ID expired on 31/12/2025. Please request a valid, unexpired ID to continue.'</t>
+          <t>Document type governs: Diplomatic ID is exception-routed to Back Office Fulfilment approval.</t>
         </is>
       </c>
       <c r="AG45" s="13" t="inlineStr">
@@ -8051,7 +8043,7 @@
       </c>
       <c r="AH45" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record.</t>
+          <t>Original demo data: customers.json, identity-documents.json</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8055,7 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>CUST-3042</t>
+          <t>CUST-3041</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr">
@@ -8078,27 +8070,27 @@
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>Nadia Hany Farouk Mansour</t>
+          <t>Omar Samer Khalil Al-Hamwi</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>Nadia</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Hany Farouk</t>
+          <t>Samer Khalil</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>Mansour</t>
+          <t>Al-Hamwi</t>
         </is>
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>Egyptian</t>
+          <t>Syrian</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr">
@@ -8113,21 +8105,25 @@
       </c>
       <c r="L46" s="13" t="inlineStr">
         <is>
-          <t>29210081800042</t>
-        </is>
-      </c>
-      <c r="M46" s="13" t="inlineStr"/>
+          <t>28808076000041</t>
+        </is>
+      </c>
+      <c r="M46" s="13" t="inlineStr">
+        <is>
+          <t>31/12/2025</t>
+        </is>
+      </c>
       <c r="N46" s="13" t="inlineStr">
         <is>
-          <t>10/10/1992</t>
+          <t>30/08/1988</t>
         </is>
       </c>
       <c r="O46" s="13" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="P46" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q46" s="13" t="inlineStr">
@@ -8142,14 +8138,14 @@
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
-          <t>+97455513028</t>
+          <t>+97455513027</t>
         </is>
       </c>
       <c r="T46" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U46" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V46" s="13" t="n">
         <v>0</v>
@@ -8183,7 +8179,7 @@
       </c>
       <c r="AD46" s="13" t="inlineStr">
         <is>
-          <t>Expat whose identity document has NO expiry date on file.</t>
+          <t>Expat whose QID EXPIRED on 31/12/2025.</t>
         </is>
       </c>
       <c r="AE46" s="13" t="inlineStr">
@@ -8193,7 +8189,7 @@
       </c>
       <c r="AF46" s="13" t="inlineStr">
         <is>
-          <t>ID Validity = approval-routing (manual validity check). Not a pass - the app never confirms an ID it cannot verify.</t>
+          <t>ID Validity hard-stop: 'This ID expired on 31/12/2025. Please request a valid, unexpired ID to continue.'</t>
         </is>
       </c>
       <c r="AG46" s="13" t="inlineStr">
@@ -8215,7 +8211,7 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>CUST-3043</t>
+          <t>CUST-3042</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">
@@ -8230,27 +8226,27 @@
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>Ravi Shankar Menon</t>
+          <t>Nadia Hany Farouk Mansour</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>Ravi</t>
+          <t>Nadia</t>
         </is>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Shankar</t>
+          <t>Hany Farouk</t>
         </is>
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
-          <t>Menon</t>
+          <t>Mansour</t>
         </is>
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>Indian</t>
+          <t>Egyptian</t>
         </is>
       </c>
       <c r="J47" s="13" t="inlineStr">
@@ -8265,25 +8261,21 @@
       </c>
       <c r="L47" s="13" t="inlineStr">
         <is>
-          <t>28912035600043</t>
-        </is>
-      </c>
-      <c r="M47" s="13" t="inlineStr">
-        <is>
-          <t>30/04/2030</t>
-        </is>
-      </c>
+          <t>29210081800042</t>
+        </is>
+      </c>
+      <c r="M47" s="13" t="inlineStr"/>
       <c r="N47" s="13" t="inlineStr">
         <is>
-          <t>15/12/1989</t>
+          <t>10/10/1992</t>
         </is>
       </c>
       <c r="O47" s="13" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="P47" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q47" s="13" t="inlineStr">
@@ -8293,12 +8285,12 @@
       </c>
       <c r="R47" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="S47" s="13" t="inlineStr">
         <is>
-          <t>+97455513029</t>
+          <t>+97455513028</t>
         </is>
       </c>
       <c r="T47" s="13" t="n">
@@ -8318,7 +8310,7 @@
       </c>
       <c r="Y47" s="13" t="inlineStr">
         <is>
-          <t>security</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z47" s="13" t="inlineStr">
@@ -8339,7 +8331,7 @@
       </c>
       <c r="AD47" s="13" t="inlineStr">
         <is>
-          <t>Expat on the corporate SECURITY blacklist.</t>
+          <t>Expat whose identity document has NO expiry date on file.</t>
         </is>
       </c>
       <c r="AE47" s="13" t="inlineStr">
@@ -8349,7 +8341,7 @@
       </c>
       <c r="AF47" s="13" t="inlineStr">
         <is>
-          <t>Security Check hard-stop; interaction ends at the counter (no prepaid fallback).</t>
+          <t>ID Validity = approval-routing (manual validity check). Not a pass - the app never confirms an ID it cannot verify.</t>
         </is>
       </c>
       <c r="AG47" s="13" t="inlineStr">
@@ -8371,7 +8363,7 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>CUST-3044</t>
+          <t>CUST-3043</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
@@ -8386,32 +8378,32 @@
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>Saeed Abdullah Nasser Al-Mohannadi</t>
+          <t>Ravi Shankar Menon</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>Saeed</t>
+          <t>Ravi</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Abdullah Nasser</t>
+          <t>Shankar</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Al-Mohannadi</t>
+          <t>Menon</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Indian</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K48" s="13" t="inlineStr">
@@ -8421,21 +8413,21 @@
       </c>
       <c r="L48" s="13" t="inlineStr">
         <is>
-          <t>30806063400044</t>
+          <t>28912035600043</t>
         </is>
       </c>
       <c r="M48" s="13" t="inlineStr">
         <is>
-          <t>31/03/2031</t>
+          <t>30/04/2030</t>
         </is>
       </c>
       <c r="N48" s="13" t="inlineStr">
         <is>
-          <t>01/06/2008</t>
+          <t>15/12/1989</t>
         </is>
       </c>
       <c r="O48" s="13" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P48" s="13" t="inlineStr">
         <is>
@@ -8449,12 +8441,12 @@
       </c>
       <c r="R48" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
-          <t>+97455513030</t>
+          <t>+97455513029</t>
         </is>
       </c>
       <c r="T48" s="13" t="n">
@@ -8474,7 +8466,7 @@
       </c>
       <c r="Y48" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>security</t>
         </is>
       </c>
       <c r="Z48" s="13" t="inlineStr">
@@ -8495,17 +8487,17 @@
       </c>
       <c r="AD48" s="13" t="inlineStr">
         <is>
-          <t>Qatari aged 18 (turned 18 on 01/06/2026) - age boundary.</t>
+          <t>Expat on the corporate SECURITY blacklist.</t>
         </is>
       </c>
       <c r="AE48" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid</t>
+          <t>Any new connection</t>
         </is>
       </c>
       <c r="AF48" s="13" t="inlineStr">
         <is>
-          <t>Age Check passes at 18 ('Customer's age is 18 years'); under 18 is a hard stop.</t>
+          <t>Security Check hard-stop; interaction ends at the counter (no prepaid fallback).</t>
         </is>
       </c>
       <c r="AG48" s="13" t="inlineStr">
@@ -8527,7 +8519,7 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>CUST-3045</t>
+          <t>CUST-3044</t>
         </is>
       </c>
       <c r="C49" s="14" t="inlineStr">
@@ -8542,60 +8534,60 @@
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>Eva Maria Mueller</t>
+          <t>Saeed Abdullah Nasser Al-Mohannadi</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>Eva</t>
+          <t>Saeed</t>
         </is>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Maria</t>
+          <t>Abdullah Nasser</t>
         </is>
       </c>
       <c r="H49" s="13" t="inlineStr">
         <is>
-          <t>Mueller</t>
+          <t>Al-Mohannadi</t>
         </is>
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>Diplomatic</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>Diplomatic ID</t>
+          <t>QID</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
         <is>
-          <t>DIP-QA-005100</t>
+          <t>30806063400044</t>
         </is>
       </c>
       <c r="M49" s="13" t="inlineStr">
         <is>
-          <t>31/12/2030</t>
+          <t>31/03/2031</t>
         </is>
       </c>
       <c r="N49" s="13" t="inlineStr">
         <is>
-          <t>18/03/1980</t>
+          <t>01/06/2008</t>
         </is>
       </c>
       <c r="O49" s="13" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="P49" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q49" s="13" t="inlineStr">
@@ -8605,12 +8597,12 @@
       </c>
       <c r="R49" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
-          <t>+97455513031</t>
+          <t>+97455513030</t>
         </is>
       </c>
       <c r="T49" s="13" t="n">
@@ -8651,7 +8643,7 @@
       </c>
       <c r="AD49" s="13" t="inlineStr">
         <is>
-          <t>German diplomat, valid Diplomatic ID, clean record.</t>
+          <t>Qatari aged 18 (turned 18 on 01/06/2026) - age boundary.</t>
         </is>
       </c>
       <c r="AE49" s="13" t="inlineStr">
@@ -8661,7 +8653,7 @@
       </c>
       <c r="AF49" s="13" t="inlineStr">
         <is>
-          <t>Diplomatic ID is exception-routed -&gt; Back Office Fulfilment approval workflow; no other block.</t>
+          <t>Age Check passes at 18 ('Customer's age is 18 years'); under 18 is a hard stop.</t>
         </is>
       </c>
       <c r="AG49" s="13" t="inlineStr">
@@ -8683,7 +8675,7 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>CUST-3046</t>
+          <t>CUST-3045</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
@@ -8698,65 +8690,65 @@
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>Bilal Ahmed Raza Siddiqui</t>
+          <t>Eva Maria Mueller</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr">
         <is>
-          <t>Bilal</t>
+          <t>Eva</t>
         </is>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Ahmed Raza</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Siddiqui</t>
+          <t>Mueller</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Pakistani</t>
+          <t>German</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>Expat (QID)</t>
+          <t>Diplomatic</t>
         </is>
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>QID</t>
+          <t>Diplomatic ID</t>
         </is>
       </c>
       <c r="L50" s="13" t="inlineStr">
         <is>
-          <t>28311058600046</t>
+          <t>DIP-QA-005100</t>
         </is>
       </c>
       <c r="M50" s="13" t="inlineStr">
         <is>
-          <t>28/02/2030</t>
+          <t>31/12/2030</t>
         </is>
       </c>
       <c r="N50" s="13" t="inlineStr">
         <is>
-          <t>11/11/1983</t>
+          <t>18/03/1980</t>
         </is>
       </c>
       <c r="O50" s="13" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="P50" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q50" s="13" t="inlineStr">
         <is>
-          <t>Consumer (HRN)</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="R50" s="13" t="inlineStr">
@@ -8766,14 +8758,14 @@
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
-          <t>+97455513032</t>
+          <t>+97455513031</t>
         </is>
       </c>
       <c r="T50" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U50" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V50" s="13" t="n">
         <v>0</v>
@@ -8786,12 +8778,12 @@
       </c>
       <c r="Y50" s="13" t="inlineStr">
         <is>
-          <t>collections</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z50" s="13" t="inlineStr">
         <is>
-          <t>HRN</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="AA50" s="13" t="inlineStr"/>
@@ -8807,17 +8799,17 @@
       </c>
       <c r="AD50" s="13" t="inlineStr">
         <is>
-          <t>Expat with a collections blacklist (dues) - postpaid blocked, prepaid available. HRN: nationality is on the VFQ list -&gt; QAR 100 advance, credit limit 50.</t>
+          <t>German diplomat, valid Diplomatic ID, clean record.</t>
         </is>
       </c>
       <c r="AE50" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid (soft-stop); New Prepaid</t>
+          <t>New Postpaid</t>
         </is>
       </c>
       <c r="AF50" s="13" t="inlineStr">
         <is>
-          <t>Collections Check soft-stop (same shape as CUST-1004 for an expat).</t>
+          <t>Diplomatic ID is exception-routed -&gt; Back Office Fulfilment approval workflow; no other block.</t>
         </is>
       </c>
       <c r="AG50" s="13" t="inlineStr">
@@ -8839,7 +8831,7 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>CUST-3072</t>
+          <t>CUST-3046</t>
         </is>
       </c>
       <c r="C51" s="14" t="inlineStr">
@@ -8854,27 +8846,27 @@
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>Rohan Vikram Mehta</t>
+          <t>Bilal Ahmed Raza Siddiqui</t>
         </is>
       </c>
       <c r="F51" s="13" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>Bilal</t>
         </is>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Vikram</t>
+          <t>Ahmed Raza</t>
         </is>
       </c>
       <c r="H51" s="13" t="inlineStr">
         <is>
-          <t>Mehta</t>
+          <t>Siddiqui</t>
         </is>
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>Indian</t>
+          <t>Pakistani</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
@@ -8889,21 +8881,21 @@
       </c>
       <c r="L51" s="13" t="inlineStr">
         <is>
-          <t>28504042200072</t>
+          <t>28311058600046</t>
         </is>
       </c>
       <c r="M51" s="13" t="inlineStr">
         <is>
-          <t>30/09/2030</t>
+          <t>28/02/2030</t>
         </is>
       </c>
       <c r="N51" s="13" t="inlineStr">
         <is>
-          <t>04/04/1985</t>
+          <t>11/11/1983</t>
         </is>
       </c>
       <c r="O51" s="13" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="P51" s="13" t="inlineStr">
         <is>
@@ -8912,7 +8904,7 @@
       </c>
       <c r="Q51" s="13" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Consumer (HRN)</t>
         </is>
       </c>
       <c r="R51" s="13" t="inlineStr">
@@ -8922,14 +8914,14 @@
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
-          <t>+97455513048</t>
+          <t>+97455513032</t>
         </is>
       </c>
       <c r="T51" s="13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U51" s="13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V51" s="13" t="n">
         <v>0</v>
@@ -8942,12 +8934,12 @@
       </c>
       <c r="Y51" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>collections</t>
         </is>
       </c>
       <c r="Z51" s="13" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>HRN</t>
         </is>
       </c>
       <c r="AA51" s="13" t="inlineStr"/>
@@ -8963,17 +8955,17 @@
       </c>
       <c r="AD51" s="13" t="inlineStr">
         <is>
-          <t>Indian expat on a valid QID already holding 5 active postpaid lines - the expat absolute maximum.</t>
+          <t>Expat with a collections blacklist (dues) - postpaid blocked, prepaid available. HRN: nationality is on the VFQ list -&gt; QAR 100 advance, credit limit 50.</t>
         </is>
       </c>
       <c r="AE51" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid</t>
+          <t>New Postpaid (soft-stop); New Prepaid</t>
         </is>
       </c>
       <c r="AF51" s="13" t="inlineStr">
         <is>
-          <t>Active Lines HARD STOP (BR-288): 'Expat maximum of 5 postpaid mobile lines reached (5 active)'. Every other check passes; the order cannot proceed (no approval route, unlike the Qatari 5+ case).</t>
+          <t>Collections Check soft-stop (same shape as CUST-1004 for an expat).</t>
         </is>
       </c>
       <c r="AG51" s="13" t="inlineStr">
@@ -8995,7 +8987,7 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>CUST-3073</t>
+          <t>CUST-3072</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
@@ -9010,27 +9002,27 @@
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>Walid Nabil Hassan Al-Zoubi</t>
+          <t>Rohan Vikram Mehta</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>Walid</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Nabil Hassan</t>
+          <t>Vikram</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>Al-Zoubi</t>
+          <t>Mehta</t>
         </is>
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>Jordanian</t>
+          <t>Indian</t>
         </is>
       </c>
       <c r="J52" s="13" t="inlineStr">
@@ -9045,17 +9037,17 @@
       </c>
       <c r="L52" s="13" t="inlineStr">
         <is>
-          <t>28509034500073</t>
+          <t>28504042200072</t>
         </is>
       </c>
       <c r="M52" s="13" t="inlineStr">
         <is>
-          <t>30/06/2030</t>
+          <t>30/09/2030</t>
         </is>
       </c>
       <c r="N52" s="13" t="inlineStr">
         <is>
-          <t>03/09/1985</t>
+          <t>04/04/1985</t>
         </is>
       </c>
       <c r="O52" s="13" t="n">
@@ -9073,19 +9065,19 @@
       </c>
       <c r="R52" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
-          <t>+97455513049</t>
+          <t>+97455513048</t>
         </is>
       </c>
       <c r="T52" s="13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U52" s="13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V52" s="13" t="n">
         <v>0</v>
@@ -9098,7 +9090,7 @@
       </c>
       <c r="Y52" s="13" t="inlineStr">
         <is>
-          <t>collections</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z52" s="13" t="inlineStr">
@@ -9119,7 +9111,7 @@
       </c>
       <c r="AD52" s="13" t="inlineStr">
         <is>
-          <t>Expat flagged on the collections blacklist but owing QAR 0 (no unpaid bill on file) - the flag alone is not a block.</t>
+          <t>Indian expat on a valid QID already holding 5 active postpaid lines - the expat absolute maximum.</t>
         </is>
       </c>
       <c r="AE52" s="13" t="inlineStr">
@@ -9129,7 +9121,7 @@
       </c>
       <c r="AF52" s="13" t="inlineStr">
         <is>
-          <t>Collections Check PASSES ('No collections block on this account'): a collections block needs an outstanding balance above QAR 0 (VFQ business, 02/10/2026). Contrast CUST-3046, same flag with an unpaid bill -&gt; soft-stop.</t>
+          <t>Active Lines HARD STOP (BR-288): 'Expat maximum of 5 postpaid mobile lines reached (5 active)'. Every other check passes; the order cannot proceed (no approval route, unlike the Qatari 5+ case).</t>
         </is>
       </c>
       <c r="AG52" s="13" t="inlineStr">
@@ -9151,7 +9143,7 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>CUST-3090</t>
+          <t>CUST-3073</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
@@ -9166,32 +9158,32 @@
       </c>
       <c r="E53" s="13" t="inlineStr">
         <is>
-          <t>Maryam Ahmed Abdulla Al-Sulaiti</t>
+          <t>Walid Nabil Hassan Al-Zoubi</t>
         </is>
       </c>
       <c r="F53" s="13" t="inlineStr">
         <is>
-          <t>Maryam</t>
+          <t>Walid</t>
         </is>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Ahmed Abdulla</t>
+          <t>Nabil Hassan</t>
         </is>
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Al-Sulaiti</t>
+          <t>Al-Zoubi</t>
         </is>
       </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Jordanian</t>
         </is>
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
@@ -9201,25 +9193,25 @@
       </c>
       <c r="L53" s="13" t="inlineStr">
         <is>
-          <t>31403153400090</t>
+          <t>28509034500073</t>
         </is>
       </c>
       <c r="M53" s="13" t="inlineStr">
         <is>
-          <t>31/03/2030</t>
+          <t>30/06/2030</t>
         </is>
       </c>
       <c r="N53" s="13" t="inlineStr">
         <is>
-          <t>15/03/2014</t>
+          <t>03/09/1985</t>
         </is>
       </c>
       <c r="O53" s="13" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="P53" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q53" s="13" t="inlineStr">
@@ -9234,14 +9226,14 @@
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
-          <t>+97455513055</t>
+          <t>+97455513049</t>
         </is>
       </c>
       <c r="T53" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U53" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V53" s="13" t="n">
         <v>0</v>
@@ -9254,7 +9246,7 @@
       </c>
       <c r="Y53" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>collections</t>
         </is>
       </c>
       <c r="Z53" s="13" t="inlineStr">
@@ -9275,17 +9267,17 @@
       </c>
       <c r="AD53" s="13" t="inlineStr">
         <is>
-          <t>Qatari aged 12 (under 18), no lines: a family member who can be added as the ACTUAL USER of a parent's postpaid line.</t>
+          <t>Expat flagged on the collections blacklist but owing QAR 0 (no unpaid bill on file) - the flag alone is not a block.</t>
         </is>
       </c>
       <c r="AE53" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid (Actual User step)</t>
+          <t>New Postpaid</t>
         </is>
       </c>
       <c r="AF53" s="13" t="inlineStr">
         <is>
-          <t>Under 18, so the Actual User step accepts her; the age rule is the only check (Number of Connections, HRN and the Collections / Grey List / Security blacklists are not run for an actual user). Anyone 18 or older is refused there.</t>
+          <t>Collections Check PASSES ('No collections block on this account'): a collections block needs an outstanding balance above QAR 0 (VFQ business, 02/10/2026). Contrast CUST-3046, same flag with an unpaid bill -&gt; soft-stop.</t>
         </is>
       </c>
       <c r="AG53" s="13" t="inlineStr">
@@ -9300,44 +9292,44 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>TC-053</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>CUST-9001</t>
-        </is>
-      </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>In app - original</t>
-        </is>
-      </c>
-      <c r="D54" s="12" t="inlineStr">
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>CUST-3090</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>In app - added 02/10/2026</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>6 Eligibility gates</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
         <is>
-          <t>Rashid Nasser Hamad Al-Naimi</t>
+          <t>Maryam Ahmed Abdulla Al-Sulaiti</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>Rashid</t>
+          <t>Maryam</t>
         </is>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Nasser Hamad</t>
+          <t>Ahmed Abdulla</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>Al-Naimi</t>
+          <t>Al-Sulaiti</t>
         </is>
       </c>
       <c r="I54" s="13" t="inlineStr">
@@ -9352,30 +9344,30 @@
       </c>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>QID / Passport</t>
+          <t>QID</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
         <is>
-          <t>12345678910 / P1234567</t>
+          <t>31403153400090</t>
         </is>
       </c>
       <c r="M54" s="13" t="inlineStr">
         <is>
-          <t>30/11/2029 / 30/11/2029</t>
+          <t>31/03/2030</t>
         </is>
       </c>
       <c r="N54" s="13" t="inlineStr">
         <is>
-          <t>20/05/2010</t>
+          <t>15/03/2014</t>
         </is>
       </c>
       <c r="O54" s="13" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="P54" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q54" s="13" t="inlineStr">
@@ -9385,12 +9377,12 @@
       </c>
       <c r="R54" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
-          <t>+97450009001</t>
+          <t>+97455513055</t>
         </is>
       </c>
       <c r="T54" s="13" t="n">
@@ -9431,17 +9423,17 @@
       </c>
       <c r="AD54" s="13" t="inlineStr">
         <is>
-          <t>QA test user, Qatari, age 16 (under 18). Holds both a QID and a Passport document.</t>
+          <t>Qatari aged 12 (under 18), no lines: a family member who can be added as the ACTUAL USER of a parent's postpaid line.</t>
         </is>
       </c>
       <c r="AE54" s="13" t="inlineStr">
         <is>
-          <t>Any new connection</t>
+          <t>New Postpaid (Actual User step)</t>
         </is>
       </c>
       <c r="AF54" s="13" t="inlineStr">
         <is>
-          <t>Age Check = HARD STOP for an under-18 applicant (02/10/2026): the connection cannot proceed.</t>
+          <t>Under 18, so the Actual User step accepts her; the age rule is the only check (Number of Connections, HRN and the Collections / Grey List / Security blacklists are not run for an actual user). Anyone 18 or older is refused there.</t>
         </is>
       </c>
       <c r="AG54" s="13" t="inlineStr">
@@ -9451,83 +9443,83 @@
       </c>
       <c r="AH54" s="13" t="inlineStr">
         <is>
-          <t>Original demo data: customers.json, identity-documents.json</t>
+          <t>Synthetic record.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="14" t="inlineStr">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>TC-054</t>
         </is>
       </c>
-      <c r="B55" s="14" t="inlineStr">
-        <is>
-          <t>CUST-3051</t>
-        </is>
-      </c>
-      <c r="C55" s="14" t="inlineStr">
-        <is>
-          <t>In app - added 02/10/2026</t>
-        </is>
-      </c>
-      <c r="D55" s="14" t="inlineStr">
-        <is>
-          <t>7 Existing-service journeys</t>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>CUST-9001</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>In app - original</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>6 Eligibility gates</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
         <is>
-          <t>Tamer Mahmoud Hosni Abdelaziz</t>
+          <t>Rashid Nasser Hamad Al-Naimi</t>
         </is>
       </c>
       <c r="F55" s="13" t="inlineStr">
         <is>
-          <t>Tamer</t>
+          <t>Rashid</t>
         </is>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Mahmoud Hosni</t>
+          <t>Nasser Hamad</t>
         </is>
       </c>
       <c r="H55" s="13" t="inlineStr">
         <is>
-          <t>Abdelaziz</t>
+          <t>Al-Naimi</t>
         </is>
       </c>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>Egyptian</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>Expat (QID)</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>QID</t>
+          <t>QID / Passport</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
         <is>
-          <t>28506081800051</t>
+          <t>12345678910 / P1234567</t>
         </is>
       </c>
       <c r="M55" s="13" t="inlineStr">
         <is>
-          <t>31/05/2030</t>
+          <t>30/11/2029 / 30/11/2029</t>
         </is>
       </c>
       <c r="N55" s="13" t="inlineStr">
         <is>
-          <t>06/06/1985</t>
+          <t>20/05/2010</t>
         </is>
       </c>
       <c r="O55" s="13" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="P55" s="13" t="inlineStr">
         <is>
@@ -9541,19 +9533,19 @@
       </c>
       <c r="R55" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
-          <t>+97455513033</t>
+          <t>+97450009001</t>
         </is>
       </c>
       <c r="T55" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U55" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V55" s="13" t="n">
         <v>0</v>
@@ -9587,27 +9579,27 @@
       </c>
       <c r="AD55" s="13" t="inlineStr">
         <is>
-          <t>Existing postpaid customer needing a SIM swap (lost SIM - chargeable) and an eSIM line.</t>
+          <t>QA test user, Qatari, age 16 (under 18). Holds both a QID and a Passport document.</t>
         </is>
       </c>
       <c r="AE55" s="13" t="inlineStr">
         <is>
-          <t>SIM Swap queue; Customer 360 Mobile section</t>
+          <t>Any new connection</t>
         </is>
       </c>
       <c r="AF55" s="13" t="inlineStr">
         <is>
-          <t>BR-056: Lost SIM is chargeable; eSIM-to-eSIM free; damaged SIM free. ID verification adds a third MOI-match step.</t>
+          <t>Age Check = HARD STOP for an under-18 applicant (02/10/2026): the connection cannot proceed.</t>
         </is>
       </c>
       <c r="AG55" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12350, VFQ12352, VFQ12354, VFQ12355, VFQ12357</t>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
         </is>
       </c>
       <c r="AH55" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record.</t>
+          <t>Original demo data: customers.json, identity-documents.json</t>
         </is>
       </c>
     </row>
@@ -9619,7 +9611,7 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>CUST-3052</t>
+          <t>CUST-3051</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
@@ -9634,32 +9626,32 @@
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>Aisha Mohammed Al-Suwaidi</t>
+          <t>Tamer Mahmoud Hosni Abdelaziz</t>
         </is>
       </c>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>Aisha</t>
+          <t>Tamer</t>
         </is>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Mohammed</t>
+          <t>Mahmoud Hosni</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t>Al-Suwaidi</t>
+          <t>Abdelaziz</t>
         </is>
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Egyptian</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K56" s="13" t="inlineStr">
@@ -9669,25 +9661,25 @@
       </c>
       <c r="L56" s="13" t="inlineStr">
         <is>
-          <t>28707063400052</t>
+          <t>28506081800051</t>
         </is>
       </c>
       <c r="M56" s="13" t="inlineStr">
         <is>
-          <t>31/08/2030</t>
+          <t>31/05/2030</t>
         </is>
       </c>
       <c r="N56" s="13" t="inlineStr">
         <is>
-          <t>25/07/1987</t>
+          <t>06/06/1985</t>
         </is>
       </c>
       <c r="O56" s="13" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="P56" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q56" s="13" t="inlineStr">
@@ -9702,7 +9694,7 @@
       </c>
       <c r="S56" s="13" t="inlineStr">
         <is>
-          <t>+97455513034</t>
+          <t>+97455513033</t>
         </is>
       </c>
       <c r="T56" s="13" t="n">
@@ -9733,7 +9725,7 @@
       <c r="AA56" s="13" t="inlineStr"/>
       <c r="AB56" s="13" t="inlineStr">
         <is>
-          <t>Loyalty (existing)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="AC56" s="13" t="inlineStr">
@@ -9743,22 +9735,22 @@
       </c>
       <c r="AD56" s="13" t="inlineStr">
         <is>
-          <t>Postpaid customer with a device instalment (Galaxy S24, 12 months) and 8 months of the 12-month lock-in completed.</t>
+          <t>Existing postpaid customer needing a SIM swap (lost SIM - chargeable) and an eSIM line.</t>
         </is>
       </c>
       <c r="AE56" s="13" t="inlineStr">
         <is>
-          <t>Customer 360; Disconnection / penalty view; Device Installment</t>
+          <t>SIM Swap queue; Customer 360 Mobile section</t>
         </is>
       </c>
       <c r="AF56" s="13" t="inlineStr">
         <is>
-          <t>Lock-in not complete -&gt; disconnection fee = QR 80 x remaining months (lock-in rule in ruleEngine.ts).</t>
+          <t>BR-056: Lost SIM is chargeable; eSIM-to-eSIM free; damaged SIM free. ID verification adds a third MOI-match step.</t>
         </is>
       </c>
       <c r="AG56" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12343, VFQ12344, VFQ12345, VFQ12346, VFQ12347, VFQ12348, VFQ12349, VFQ12350, VFQ12351, VFQ12352, VFQ12353, VFQ12354, VFQ12355, VFQ12356, VFQ12357, VFQ12358, VFQ12359, VFQ12362, VFQ12363, VFQ12365, VFQ12366</t>
+          <t>VFQ12341, VFQ12350, VFQ12352, VFQ12354, VFQ12355, VFQ12357</t>
         </is>
       </c>
       <c r="AH56" s="13" t="inlineStr">
@@ -9775,7 +9767,7 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>CUST-3053</t>
+          <t>CUST-3052</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -9790,22 +9782,22 @@
       </c>
       <c r="E57" s="13" t="inlineStr">
         <is>
-          <t>Faisal Hamad Saud Al-Rumaihi</t>
+          <t>Aisha Mohammed Al-Suwaidi</t>
         </is>
       </c>
       <c r="F57" s="13" t="inlineStr">
         <is>
-          <t>Faisal</t>
+          <t>Aisha</t>
         </is>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>Hamad Saud</t>
+          <t>Mohammed</t>
         </is>
       </c>
       <c r="H57" s="13" t="inlineStr">
         <is>
-          <t>Al-Rumaihi</t>
+          <t>Al-Suwaidi</t>
         </is>
       </c>
       <c r="I57" s="13" t="inlineStr">
@@ -9825,25 +9817,25 @@
       </c>
       <c r="L57" s="13" t="inlineStr">
         <is>
-          <t>28808063400053</t>
+          <t>28707063400052</t>
         </is>
       </c>
       <c r="M57" s="13" t="inlineStr">
         <is>
-          <t>31/03/2030</t>
+          <t>31/08/2030</t>
         </is>
       </c>
       <c r="N57" s="13" t="inlineStr">
         <is>
-          <t>19/08/1988</t>
+          <t>25/07/1987</t>
         </is>
       </c>
       <c r="O57" s="13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P57" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q57" s="13" t="inlineStr">
@@ -9858,7 +9850,7 @@
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
-          <t>+97455513035</t>
+          <t>+97455513034</t>
         </is>
       </c>
       <c r="T57" s="13" t="n">
@@ -9899,22 +9891,22 @@
       </c>
       <c r="AD57" s="13" t="inlineStr">
         <is>
-          <t>Qatari with a GigaHome 5G FWA outdoor line plus 1 postpaid line (cross-sell target).</t>
+          <t>Postpaid customer with a device instalment (Galaxy S24, 12 months) and 8 months of the 12-month lock-in completed.</t>
         </is>
       </c>
       <c r="AE57" s="13" t="inlineStr">
         <is>
-          <t>FWA; Fixed Line; Customer 360</t>
+          <t>Customer 360; Disconnection / penalty view; Device Installment</t>
         </is>
       </c>
       <c r="AF57" s="13" t="inlineStr">
         <is>
-          <t>Existing multi-product customer; FWA appointment booking and serial-number check apply.</t>
+          <t>Lock-in not complete -&gt; disconnection fee = QR 80 x remaining months (lock-in rule in ruleEngine.ts).</t>
         </is>
       </c>
       <c r="AG57" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12343, VFQ12344, VFQ12345</t>
+          <t>VFQ12341, VFQ12342, VFQ12343, VFQ12344, VFQ12345, VFQ12346, VFQ12347, VFQ12348, VFQ12349, VFQ12350, VFQ12351, VFQ12352, VFQ12353, VFQ12354, VFQ12355, VFQ12356, VFQ12357, VFQ12358, VFQ12359, VFQ12362, VFQ12363, VFQ12365, VFQ12366</t>
         </is>
       </c>
       <c r="AH57" s="13" t="inlineStr">
@@ -9931,7 +9923,7 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>CUST-3054</t>
+          <t>CUST-3053</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
@@ -9946,22 +9938,22 @@
       </c>
       <c r="E58" s="13" t="inlineStr">
         <is>
-          <t>Zainab Ibrahim Khalid Al-Hashemi</t>
+          <t>Faisal Hamad Saud Al-Rumaihi</t>
         </is>
       </c>
       <c r="F58" s="13" t="inlineStr">
         <is>
-          <t>Zainab</t>
+          <t>Faisal</t>
         </is>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>Ibrahim Khalid</t>
+          <t>Hamad Saud</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t>Al-Hashemi</t>
+          <t>Al-Rumaihi</t>
         </is>
       </c>
       <c r="I58" s="13" t="inlineStr">
@@ -9981,25 +9973,25 @@
       </c>
       <c r="L58" s="13" t="inlineStr">
         <is>
-          <t>29108063400054</t>
+          <t>28808063400053</t>
         </is>
       </c>
       <c r="M58" s="13" t="inlineStr">
         <is>
-          <t>30/11/2030</t>
+          <t>31/03/2030</t>
         </is>
       </c>
       <c r="N58" s="13" t="inlineStr">
         <is>
-          <t>14/08/1991</t>
+          <t>19/08/1988</t>
         </is>
       </c>
       <c r="O58" s="13" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="P58" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q58" s="13" t="inlineStr">
@@ -10009,22 +10001,22 @@
       </c>
       <c r="R58" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
-          <t>+97455513036</t>
+          <t>+97455513035</t>
         </is>
       </c>
       <c r="T58" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U58" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V58" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W58" s="13" t="n">
         <v>0</v>
@@ -10055,22 +10047,22 @@
       </c>
       <c r="AD58" s="13" t="inlineStr">
         <is>
-          <t>High-value Qatari with multi-SIM / iWatch lines; high-value retention target.</t>
+          <t>Qatari with a GigaHome 5G FWA outdoor line plus 1 postpaid line (cross-sell target).</t>
         </is>
       </c>
       <c r="AE58" s="13" t="inlineStr">
         <is>
-          <t>Retention; Customer 360; Multi-SIM</t>
+          <t>FWA; Fixed Line; Customer 360</t>
         </is>
       </c>
       <c r="AF58" s="13" t="inlineStr">
         <is>
-          <t>Premium / Retention journeys; multi-SIM sequence numbers and monthly fees apply.</t>
+          <t>Existing multi-product customer; FWA appointment booking and serial-number check apply.</t>
         </is>
       </c>
       <c r="AG58" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12343, VFQ12344, VFQ12345, VFQ12346, VFQ12347, VFQ12348, VFQ12349, VFQ12350, VFQ12351, VFQ12352, VFQ12353, VFQ12354, VFQ12355, VFQ12356, VFQ12357, VFQ12358, VFQ12359, VFQ12362, VFQ12363, VFQ12365, VFQ12366</t>
+          <t>VFQ12341, VFQ12343, VFQ12344, VFQ12345</t>
         </is>
       </c>
       <c r="AH58" s="13" t="inlineStr">
@@ -10087,7 +10079,7 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>CUST-3061</t>
+          <t>CUST-3054</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -10097,70 +10089,70 @@
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>8 HRN &amp; ID classes</t>
+          <t>7 Existing-service journeys</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>Mizanur Abdul Karim Rahman</t>
+          <t>Zainab Ibrahim Khalid Al-Hashemi</t>
         </is>
       </c>
       <c r="F59" s="13" t="inlineStr">
         <is>
-          <t>Mizanur</t>
+          <t>Zainab</t>
         </is>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>Abdul Karim</t>
+          <t>Ibrahim Khalid</t>
         </is>
       </c>
       <c r="H59" s="13" t="inlineStr">
         <is>
-          <t>Rahman</t>
+          <t>Al-Hashemi</t>
         </is>
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>Bangladeshi</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>Expat (Passport)</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="K59" s="13" t="inlineStr">
         <is>
-          <t>Passport</t>
+          <t>QID</t>
         </is>
       </c>
       <c r="L59" s="13" t="inlineStr">
         <is>
-          <t>BN7721045</t>
+          <t>29108063400054</t>
         </is>
       </c>
       <c r="M59" s="13" t="inlineStr">
         <is>
-          <t>30/04/2031</t>
+          <t>30/11/2030</t>
         </is>
       </c>
       <c r="N59" s="13" t="inlineStr">
         <is>
-          <t>08/03/1990</t>
+          <t>14/08/1991</t>
         </is>
       </c>
       <c r="O59" s="13" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P59" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q59" s="13" t="inlineStr">
         <is>
-          <t>Consumer (HRN)</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="R59" s="13" t="inlineStr">
@@ -10170,17 +10162,17 @@
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
-          <t>+97455513037</t>
+          <t>+97455513036</t>
         </is>
       </c>
       <c r="T59" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U59" s="13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V59" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W59" s="13" t="n">
         <v>0</v>
@@ -10195,13 +10187,13 @@
       </c>
       <c r="Z59" s="13" t="inlineStr">
         <is>
-          <t>HRN</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="AA59" s="13" t="inlineStr"/>
       <c r="AB59" s="13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Loyalty (existing)</t>
         </is>
       </c>
       <c r="AC59" s="13" t="inlineStr">
@@ -10211,27 +10203,27 @@
       </c>
       <c r="AD59" s="13" t="inlineStr">
         <is>
-          <t>HRN expat on a Passport with 2 prepaid lines = Passport prepaid cap.</t>
+          <t>High-value Qatari with multi-SIM / iWatch lines; high-value retention target.</t>
         </is>
       </c>
       <c r="AE59" s="13" t="inlineStr">
         <is>
-          <t>New Prepaid (blocked); New Connection</t>
+          <t>Retention; Customer 360; Multi-SIM</t>
         </is>
       </c>
       <c r="AF59" s="13" t="inlineStr">
         <is>
-          <t>Prepaid cap 2 reached (BR-347) -&gt; line limit reached, order routed for approval; Passport is permitted on prepaid (KYC_01) so there is no ID-type routing there. HRN: on prepaid the flag is only stored (no QAR 100 advance, no message, no approval - CAM_03/CAM_04); on postpaid the QAR 100 advance and credit limit 50 apply. Passport is not offered for New Postpaid.</t>
+          <t>Premium / Retention journeys; multi-SIM sequence numbers and monthly fees apply.</t>
         </is>
       </c>
       <c r="AG59" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345</t>
+          <t>VFQ12341, VFQ12342, VFQ12343, VFQ12344, VFQ12345, VFQ12346, VFQ12347, VFQ12348, VFQ12349, VFQ12350, VFQ12351, VFQ12352, VFQ12353, VFQ12354, VFQ12355, VFQ12356, VFQ12357, VFQ12358, VFQ12359, VFQ12362, VFQ12363, VFQ12365, VFQ12366</t>
         </is>
       </c>
       <c r="AH59" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record. Nationality chosen for realism - the app reads only the HRN flag, not a nationality list.</t>
+          <t>Synthetic record.</t>
         </is>
       </c>
     </row>
@@ -10243,7 +10235,7 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>CUST-3062</t>
+          <t>CUST-3061</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
@@ -10258,56 +10250,56 @@
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>Samuel Okello Mugisha</t>
+          <t>Mizanur Abdul Karim Rahman</t>
         </is>
       </c>
       <c r="F60" s="13" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Mizanur</t>
         </is>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>Okello</t>
+          <t>Abdul Karim</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr">
         <is>
-          <t>Mugisha</t>
+          <t>Rahman</t>
         </is>
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>Ugandan</t>
+          <t>Bangladeshi</t>
         </is>
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>Expat (QID)</t>
+          <t>Expat (Passport)</t>
         </is>
       </c>
       <c r="K60" s="13" t="inlineStr">
         <is>
-          <t>QID</t>
+          <t>Passport</t>
         </is>
       </c>
       <c r="L60" s="13" t="inlineStr">
         <is>
-          <t>29207052400062</t>
+          <t>BN7721045</t>
         </is>
       </c>
       <c r="M60" s="13" t="inlineStr">
         <is>
-          <t>30/09/2030</t>
+          <t>30/04/2031</t>
         </is>
       </c>
       <c r="N60" s="13" t="inlineStr">
         <is>
-          <t>04/07/1992</t>
+          <t>08/03/1990</t>
         </is>
       </c>
       <c r="O60" s="13" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P60" s="13" t="inlineStr">
         <is>
@@ -10326,17 +10318,17 @@
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
-          <t>+97455513038</t>
+          <t>+97455513037</t>
         </is>
       </c>
       <c r="T60" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U60" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V60" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W60" s="13" t="n">
         <v>0</v>
@@ -10354,14 +10346,10 @@
           <t>HRN</t>
         </is>
       </c>
-      <c r="AA60" s="13" t="inlineStr">
-        <is>
-          <t>Gulf Logistics W.L.L.</t>
-        </is>
-      </c>
+      <c r="AA60" s="13" t="inlineStr"/>
       <c r="AB60" s="13" t="inlineStr">
         <is>
-          <t>B2B2C (-10% on Red 500)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="AC60" s="13" t="inlineStr">
@@ -10371,27 +10359,27 @@
       </c>
       <c r="AD60" s="13" t="inlineStr">
         <is>
-          <t>HRN expat (Ugandan) sponsored by Gulf Logistics W.L.L. (HRN + B2B2C), 1 postpaid line.</t>
+          <t>HRN expat on a Passport with 2 prepaid lines = Passport prepaid cap.</t>
         </is>
       </c>
       <c r="AE60" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid; FWA; Fixed Line</t>
+          <t>New Prepaid (blocked); New Connection</t>
         </is>
       </c>
       <c r="AF60" s="13" t="inlineStr">
         <is>
-          <t>Both apply: HRN advance QAR 100 AND B2B2C route (Submitted for Approval, Proof of Employment mandatory). B2B2C wins the order sub-type (orderSubType = B2B2C).</t>
+          <t>Prepaid cap 2 reached (BR-347) -&gt; line limit reached, order routed for approval; Passport is permitted on prepaid (KYC_01) so there is no ID-type routing there. HRN: on prepaid the flag is only stored (no QAR 100 advance, no message, no approval - CAM_03/CAM_04); on postpaid the QAR 100 advance and credit limit 50 apply. Passport is not offered for New Postpaid.</t>
         </is>
       </c>
       <c r="AG60" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345</t>
         </is>
       </c>
       <c r="AH60" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record.</t>
+          <t>Synthetic record. Nationality chosen for realism - the app reads only the HRN flag, not a nationality list.</t>
         </is>
       </c>
     </row>
@@ -10403,7 +10391,7 @@
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>CUST-3063</t>
+          <t>CUST-3062</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
@@ -10418,56 +10406,56 @@
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>Zahid Mehmood Butt</t>
+          <t>Samuel Okello Mugisha</t>
         </is>
       </c>
       <c r="F61" s="13" t="inlineStr">
         <is>
-          <t>Zahid</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>Mehmood</t>
+          <t>Okello</t>
         </is>
       </c>
       <c r="H61" s="13" t="inlineStr">
         <is>
-          <t>Butt</t>
+          <t>Mugisha</t>
         </is>
       </c>
       <c r="I61" s="13" t="inlineStr">
         <is>
-          <t>Pakistani</t>
+          <t>Ugandan</t>
         </is>
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>Expat (Other ID)</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K61" s="13" t="inlineStr">
         <is>
-          <t>Other ID</t>
+          <t>QID</t>
         </is>
       </c>
       <c r="L61" s="13" t="inlineStr">
         <is>
-          <t>RES-9930471</t>
+          <t>29207052400062</t>
         </is>
       </c>
       <c r="M61" s="13" t="inlineStr">
         <is>
-          <t>31/01/2030</t>
+          <t>30/09/2030</t>
         </is>
       </c>
       <c r="N61" s="13" t="inlineStr">
         <is>
-          <t>21/09/1990</t>
+          <t>04/07/1992</t>
         </is>
       </c>
       <c r="O61" s="13" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="P61" s="13" t="inlineStr">
         <is>
@@ -10481,22 +10469,22 @@
       </c>
       <c r="R61" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="S61" s="13" t="inlineStr">
         <is>
-          <t>+97455513039</t>
+          <t>+97455513038</t>
         </is>
       </c>
       <c r="T61" s="13" t="n">
         <v>1</v>
       </c>
       <c r="U61" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V61" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W61" s="13" t="n">
         <v>0</v>
@@ -10514,10 +10502,14 @@
           <t>HRN</t>
         </is>
       </c>
-      <c r="AA61" s="13" t="inlineStr"/>
+      <c r="AA61" s="13" t="inlineStr">
+        <is>
+          <t>Gulf Logistics W.L.L.</t>
+        </is>
+      </c>
       <c r="AB61" s="13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>B2B2C (-10% on Red 500)</t>
         </is>
       </c>
       <c r="AC61" s="13" t="inlineStr">
@@ -10527,27 +10519,27 @@
       </c>
       <c r="AD61" s="13" t="inlineStr">
         <is>
-          <t>HRN expat (Pakistani) holding an 'Other ID' (resident permit) with 1 prepaid line - HRN together with an exception-routed ID type.</t>
+          <t>HRN expat (Ugandan) sponsored by Gulf Logistics W.L.L. (HRN + B2B2C), 1 postpaid line.</t>
         </is>
       </c>
       <c r="AE61" s="13" t="inlineStr">
         <is>
-          <t>New Prepaid; Customer Search</t>
+          <t>New Postpaid; FWA; Fixed Line</t>
         </is>
       </c>
       <c r="AF61" s="13" t="inlineStr">
         <is>
-          <t>Other ID exception-routed to Back Office Fulfilment approval (also on prepaid: it is not one of the four permitted prepaid ID types); HRN is only stored on prepaid (no QAR 100 advance); prepaid cap not an expat-QID cap. Find by mobile/name - the ID selector has no Other ID option.</t>
+          <t>Both apply: HRN advance QAR 100 AND B2B2C route (Submitted for Approval, Proof of Employment mandatory). B2B2C wins the order sub-type (orderSubType = B2B2C).</t>
         </is>
       </c>
       <c r="AG61" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345</t>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
         </is>
       </c>
       <c r="AH61" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record. Look up via Customer Search (mobile/name); the ID selector has no Other ID option.</t>
+          <t>Synthetic record.</t>
         </is>
       </c>
     </row>
@@ -10559,7 +10551,7 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>CUST-3064</t>
+          <t>CUST-3063</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
@@ -10574,56 +10566,56 @@
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>Kyaw Zin Htet</t>
+          <t>Zahid Mehmood Butt</t>
         </is>
       </c>
       <c r="F62" s="13" t="inlineStr">
         <is>
-          <t>Kyaw</t>
+          <t>Zahid</t>
         </is>
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>Zin</t>
+          <t>Mehmood</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>Htet</t>
+          <t>Butt</t>
         </is>
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>Myanmar</t>
+          <t>Pakistani</t>
         </is>
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>Expat (QID)</t>
+          <t>Expat (Other ID)</t>
         </is>
       </c>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>QID</t>
+          <t>Other ID</t>
         </is>
       </c>
       <c r="L62" s="13" t="inlineStr">
         <is>
-          <t>28809072900064</t>
+          <t>RES-9930471</t>
         </is>
       </c>
       <c r="M62" s="13" t="inlineStr">
         <is>
-          <t>30/11/2029</t>
+          <t>31/01/2030</t>
         </is>
       </c>
       <c r="N62" s="13" t="inlineStr">
         <is>
-          <t>12/09/1988</t>
+          <t>21/09/1990</t>
         </is>
       </c>
       <c r="O62" s="13" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="P62" s="13" t="inlineStr">
         <is>
@@ -10642,17 +10634,17 @@
       </c>
       <c r="S62" s="13" t="inlineStr">
         <is>
-          <t>+97455513040</t>
+          <t>+97455513039</t>
         </is>
       </c>
       <c r="T62" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U62" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V62" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W62" s="13" t="n">
         <v>0</v>
@@ -10673,7 +10665,7 @@
       <c r="AA62" s="13" t="inlineStr"/>
       <c r="AB62" s="13" t="inlineStr">
         <is>
-          <t>Loyalty (existing)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="AC62" s="13" t="inlineStr">
@@ -10683,27 +10675,27 @@
       </c>
       <c r="AD62" s="13" t="inlineStr">
         <is>
-          <t>HRN expat (Myanmar) QID with 2 postpaid lines (AT the expat cap).</t>
+          <t>HRN expat (Pakistani) holding an 'Other ID' (resident permit) with 1 prepaid line - HRN together with an exception-routed ID type.</t>
         </is>
       </c>
       <c r="AE62" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid (3rd line)</t>
+          <t>New Prepaid; Customer Search</t>
         </is>
       </c>
       <c r="AF62" s="13" t="inlineStr">
         <is>
-          <t>Two independent gates: expat cap of 2 -&gt; approval task, AND HRN QAR 100 advance. Both must clear.</t>
+          <t>Other ID exception-routed to Back Office Fulfilment approval (also on prepaid: it is not one of the four permitted prepaid ID types); HRN is only stored on prepaid (no QAR 100 advance); prepaid cap not an expat-QID cap. Find by mobile/name - the ID selector has no Other ID option.</t>
         </is>
       </c>
       <c r="AG62" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345</t>
         </is>
       </c>
       <c r="AH62" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record.</t>
+          <t>Synthetic record. Look up via Customer Search (mobile/name); the ID selector has no Other ID option.</t>
         </is>
       </c>
     </row>
@@ -10715,7 +10707,7 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>CUST-3065</t>
+          <t>CUST-3064</t>
         </is>
       </c>
       <c r="C63" s="14" t="inlineStr">
@@ -10730,32 +10722,32 @@
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>Abdulrahman Jassim Hamad Al-Kubaisi</t>
+          <t>Kyaw Zin Htet</t>
         </is>
       </c>
       <c r="F63" s="13" t="inlineStr">
         <is>
-          <t>Abdulrahman</t>
+          <t>Kyaw</t>
         </is>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Jassim Hamad</t>
+          <t>Zin</t>
         </is>
       </c>
       <c r="H63" s="13" t="inlineStr">
         <is>
-          <t>Al-Kubaisi</t>
+          <t>Htet</t>
         </is>
       </c>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Myanmar</t>
         </is>
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>Qatari (Sawfa)</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
@@ -10765,21 +10757,21 @@
       </c>
       <c r="L63" s="13" t="inlineStr">
         <is>
-          <t>28402063400065</t>
+          <t>28809072900064</t>
         </is>
       </c>
       <c r="M63" s="13" t="inlineStr">
         <is>
-          <t>31/05/2030</t>
+          <t>30/11/2029</t>
         </is>
       </c>
       <c r="N63" s="13" t="inlineStr">
         <is>
-          <t>17/02/1984</t>
+          <t>12/09/1988</t>
         </is>
       </c>
       <c r="O63" s="13" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="P63" s="13" t="inlineStr">
         <is>
@@ -10788,7 +10780,7 @@
       </c>
       <c r="Q63" s="13" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Consumer (HRN)</t>
         </is>
       </c>
       <c r="R63" s="13" t="inlineStr">
@@ -10798,17 +10790,17 @@
       </c>
       <c r="S63" s="13" t="inlineStr">
         <is>
-          <t>+97455513041</t>
+          <t>+97455513040</t>
         </is>
       </c>
       <c r="T63" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U63" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V63" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W63" s="13" t="n">
         <v>0</v>
@@ -10823,7 +10815,7 @@
       </c>
       <c r="Z63" s="13" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>HRN</t>
         </is>
       </c>
       <c r="AA63" s="13" t="inlineStr"/>
@@ -10839,22 +10831,22 @@
       </c>
       <c r="AD63" s="13" t="inlineStr">
         <is>
-          <t>Qatari in the Sawfa category (BR-347: no prepaid restriction). 1 postpaid + 2 prepaid.</t>
+          <t>HRN expat (Myanmar) QID with 2 postpaid lines (AT the expat cap).</t>
         </is>
       </c>
       <c r="AE63" s="13" t="inlineStr">
         <is>
-          <t>New Prepaid; New Postpaid</t>
+          <t>New Postpaid (3rd line)</t>
         </is>
       </c>
       <c r="AF63" s="13" t="inlineStr">
         <is>
-          <t>No prepaid cap; postpaid 1/5. DATA ONLY: the app stores customerSubType but does not branch on Sawfa - Qatari rules already apply (Open Questions Q9).</t>
+          <t>Two independent gates: expat cap of 2 -&gt; approval task, AND HRN QAR 100 advance. Both must clear.</t>
         </is>
       </c>
       <c r="AG63" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345</t>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
         </is>
       </c>
       <c r="AH63" s="13" t="inlineStr">
@@ -10871,7 +10863,7 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>CUST-3066</t>
+          <t>CUST-3065</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
@@ -10886,22 +10878,22 @@
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>Maha Rashid Saeed Al-Ghanim</t>
+          <t>Abdulrahman Jassim Hamad Al-Kubaisi</t>
         </is>
       </c>
       <c r="F64" s="13" t="inlineStr">
         <is>
-          <t>Maha</t>
+          <t>Abdulrahman</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Rashid Saeed</t>
+          <t>Jassim Hamad</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr">
         <is>
-          <t>Al-Ghanim</t>
+          <t>Al-Kubaisi</t>
         </is>
       </c>
       <c r="I64" s="13" t="inlineStr">
@@ -10911,7 +10903,7 @@
       </c>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>Qatari (Sawfa Plus)</t>
+          <t>Qatari (Sawfa)</t>
         </is>
       </c>
       <c r="K64" s="13" t="inlineStr">
@@ -10921,25 +10913,25 @@
       </c>
       <c r="L64" s="13" t="inlineStr">
         <is>
-          <t>28704063400066</t>
+          <t>28402063400065</t>
         </is>
       </c>
       <c r="M64" s="13" t="inlineStr">
         <is>
-          <t>31/07/2030</t>
+          <t>31/05/2030</t>
         </is>
       </c>
       <c r="N64" s="13" t="inlineStr">
         <is>
-          <t>26/04/1987</t>
+          <t>17/02/1984</t>
         </is>
       </c>
       <c r="O64" s="13" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P64" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q64" s="13" t="inlineStr">
@@ -10954,17 +10946,17 @@
       </c>
       <c r="S64" s="13" t="inlineStr">
         <is>
-          <t>+97455513042</t>
+          <t>+97455513041</t>
         </is>
       </c>
       <c r="T64" s="13" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="U64" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V64" s="13" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="W64" s="13" t="n">
         <v>0</v>
@@ -10985,7 +10977,7 @@
       <c r="AA64" s="13" t="inlineStr"/>
       <c r="AB64" s="13" t="inlineStr">
         <is>
-          <t>Prepaid Welcome (-10%)</t>
+          <t>Loyalty (existing)</t>
         </is>
       </c>
       <c r="AC64" s="13" t="inlineStr">
@@ -10995,17 +10987,17 @@
       </c>
       <c r="AD64" s="13" t="inlineStr">
         <is>
-          <t>Qatari in the Sawfa Plus category with 7 prepaid lines - well past any expat cap.</t>
+          <t>Qatari in the Sawfa category (BR-347: no prepaid restriction). 1 postpaid + 2 prepaid.</t>
         </is>
       </c>
       <c r="AE64" s="13" t="inlineStr">
         <is>
-          <t>New Prepaid</t>
+          <t>New Prepaid; New Postpaid</t>
         </is>
       </c>
       <c r="AF64" s="13" t="inlineStr">
         <is>
-          <t>Qatari: prepaid cap not applied (BR-347), so an 8th prepaid line passes. DATA ONLY for the Sawfa Plus label (Q9).</t>
+          <t>No prepaid cap; postpaid 1/5. DATA ONLY: the app stores customerSubType but does not branch on Sawfa - Qatari rules already apply (Open Questions Q9).</t>
         </is>
       </c>
       <c r="AG64" s="13" t="inlineStr">
@@ -11027,7 +11019,7 @@
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>CUST-3067</t>
+          <t>CUST-3066</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
@@ -11042,52 +11034,52 @@
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>Mohamed Nabil Ibrahim Soliman</t>
+          <t>Maha Rashid Saeed Al-Ghanim</t>
         </is>
       </c>
       <c r="F65" s="13" t="inlineStr">
         <is>
-          <t>Mohamed</t>
+          <t>Maha</t>
         </is>
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>Nabil Ibrahim</t>
+          <t>Rashid Saeed</t>
         </is>
       </c>
       <c r="H65" s="13" t="inlineStr">
         <is>
-          <t>Soliman</t>
+          <t>Al-Ghanim</t>
         </is>
       </c>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>Egyptian</t>
+          <t>Qatari</t>
         </is>
       </c>
       <c r="J65" s="13" t="inlineStr">
         <is>
-          <t>Expat (Other ID)</t>
+          <t>Qatari (Sawfa Plus)</t>
         </is>
       </c>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>Other ID</t>
+          <t>QID</t>
         </is>
       </c>
       <c r="L65" s="13" t="inlineStr">
         <is>
-          <t>RES-8812045</t>
+          <t>28704063400066</t>
         </is>
       </c>
       <c r="M65" s="13" t="inlineStr">
         <is>
-          <t>31/03/2030</t>
+          <t>31/07/2030</t>
         </is>
       </c>
       <c r="N65" s="13" t="inlineStr">
         <is>
-          <t>20/12/1986</t>
+          <t>26/04/1987</t>
         </is>
       </c>
       <c r="O65" s="13" t="n">
@@ -11095,7 +11087,7 @@
       </c>
       <c r="P65" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q65" s="13" t="inlineStr">
@@ -11110,17 +11102,17 @@
       </c>
       <c r="S65" s="13" t="inlineStr">
         <is>
-          <t>+97455513043</t>
+          <t>+97455513042</t>
         </is>
       </c>
       <c r="T65" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="U65" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V65" s="13" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="W65" s="13" t="n">
         <v>0</v>
@@ -11141,7 +11133,7 @@
       <c r="AA65" s="13" t="inlineStr"/>
       <c r="AB65" s="13" t="inlineStr">
         <is>
-          <t>Loyalty (existing)</t>
+          <t>Prepaid Welcome (-10%)</t>
         </is>
       </c>
       <c r="AC65" s="13" t="inlineStr">
@@ -11151,27 +11143,27 @@
       </c>
       <c r="AD65" s="13" t="inlineStr">
         <is>
-          <t>Expat holding a resident-permit style 'Other ID' (no QID), 1 postpaid line.</t>
+          <t>Qatari in the Sawfa Plus category with 7 prepaid lines - well past any expat cap.</t>
         </is>
       </c>
       <c r="AE65" s="13" t="inlineStr">
         <is>
-          <t>Customer 360; New Postpaid</t>
+          <t>New Prepaid</t>
         </is>
       </c>
       <c r="AF65" s="13" t="inlineStr">
         <is>
-          <t>Other ID is exception-routed to Back Office Fulfilment approval. NOTE: the ID-type selector does not offer 'Other ID', so find this customer by Mobile/name in Customer Search, not by ID scan.</t>
+          <t>Qatari: prepaid cap not applied (BR-347), so an 8th prepaid line passes. DATA ONLY for the Sawfa Plus label (Q9).</t>
         </is>
       </c>
       <c r="AG65" s="13" t="inlineStr">
         <is>
-          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345</t>
         </is>
       </c>
       <c r="AH65" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record. Look up via Customer Search (mobile/name); the ID selector has no Other ID option.</t>
+          <t>Synthetic record.</t>
         </is>
       </c>
     </row>
@@ -11183,7 +11175,7 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>CUST-3068</t>
+          <t>CUST-3067</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
@@ -11198,56 +11190,56 @@
       </c>
       <c r="E66" s="13" t="inlineStr">
         <is>
-          <t>Sokha Vannak Chea</t>
+          <t>Mohamed Nabil Ibrahim Soliman</t>
         </is>
       </c>
       <c r="F66" s="13" t="inlineStr">
         <is>
-          <t>Sokha</t>
+          <t>Mohamed</t>
         </is>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>Vannak</t>
+          <t>Nabil Ibrahim</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr">
         <is>
-          <t>Chea</t>
+          <t>Soliman</t>
         </is>
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>Cambodian</t>
+          <t>Egyptian</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>Expat (QID)</t>
+          <t>Expat (Other ID)</t>
         </is>
       </c>
       <c r="K66" s="13" t="inlineStr">
         <is>
-          <t>QID</t>
+          <t>Other ID</t>
         </is>
       </c>
       <c r="L66" s="13" t="inlineStr">
         <is>
-          <t>29506011600068</t>
+          <t>RES-8812045</t>
         </is>
       </c>
       <c r="M66" s="13" t="inlineStr">
         <is>
-          <t>28/02/2030</t>
+          <t>31/03/2030</t>
         </is>
       </c>
       <c r="N66" s="13" t="inlineStr">
         <is>
-          <t>14/06/1995</t>
+          <t>20/12/1986</t>
         </is>
       </c>
       <c r="O66" s="13" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="P66" s="13" t="inlineStr">
         <is>
@@ -11256,24 +11248,24 @@
       </c>
       <c r="Q66" s="13" t="inlineStr">
         <is>
-          <t>Consumer (HRN)</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="R66" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="S66" s="13" t="inlineStr">
         <is>
-          <t>+97455513044</t>
+          <t>+97455513043</t>
         </is>
       </c>
       <c r="T66" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U66" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V66" s="13" t="n">
         <v>0</v>
@@ -11291,13 +11283,13 @@
       </c>
       <c r="Z66" s="13" t="inlineStr">
         <is>
-          <t>HRN</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="AA66" s="13" t="inlineStr"/>
       <c r="AB66" s="13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Loyalty (existing)</t>
         </is>
       </c>
       <c r="AC66" s="13" t="inlineStr">
@@ -11307,17 +11299,17 @@
       </c>
       <c r="AD66" s="13" t="inlineStr">
         <is>
-          <t>Cambodian expat on a valid QID, no lines - HRN nationality coverage.</t>
+          <t>Expat holding a resident-permit style 'Other ID' (no QID), 1 postpaid line.</t>
         </is>
       </c>
       <c r="AE66" s="13" t="inlineStr">
         <is>
-          <t>New Postpaid</t>
+          <t>Customer 360; New Postpaid</t>
         </is>
       </c>
       <c r="AF66" s="13" t="inlineStr">
         <is>
-          <t>HRN (Cambodia is on the list): QAR 100 advance and credit limit 50.</t>
+          <t>Other ID is exception-routed to Back Office Fulfilment approval. NOTE: the ID-type selector does not offer 'Other ID', so find this customer by Mobile/name in Customer Search, not by ID scan.</t>
         </is>
       </c>
       <c r="AG66" s="13" t="inlineStr">
@@ -11327,7 +11319,7 @@
       </c>
       <c r="AH66" s="13" t="inlineStr">
         <is>
-          <t>Synthetic record.</t>
+          <t>Synthetic record. Look up via Customer Search (mobile/name); the ID selector has no Other ID option.</t>
         </is>
       </c>
     </row>
@@ -11339,7 +11331,7 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>CUST-3069</t>
+          <t>CUST-3068</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
@@ -11354,27 +11346,27 @@
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>Khamla Somphone Vongsa</t>
+          <t>Sokha Vannak Chea</t>
         </is>
       </c>
       <c r="F67" s="13" t="inlineStr">
         <is>
-          <t>Khamla</t>
+          <t>Sokha</t>
         </is>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Somphone</t>
+          <t>Vannak</t>
         </is>
       </c>
       <c r="H67" s="13" t="inlineStr">
         <is>
-          <t>Vongsa</t>
+          <t>Chea</t>
         </is>
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>Laotian</t>
+          <t>Cambodian</t>
         </is>
       </c>
       <c r="J67" s="13" t="inlineStr">
@@ -11389,25 +11381,25 @@
       </c>
       <c r="L67" s="13" t="inlineStr">
         <is>
-          <t>28910041800069</t>
+          <t>29506011600068</t>
         </is>
       </c>
       <c r="M67" s="13" t="inlineStr">
         <is>
-          <t>31/12/2029</t>
+          <t>28/02/2030</t>
         </is>
       </c>
       <c r="N67" s="13" t="inlineStr">
         <is>
-          <t>02/10/1989</t>
+          <t>14/06/1995</t>
         </is>
       </c>
       <c r="O67" s="13" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="P67" s="13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Q67" s="13" t="inlineStr">
@@ -11422,7 +11414,7 @@
       </c>
       <c r="S67" s="13" t="inlineStr">
         <is>
-          <t>+97455513045</t>
+          <t>+97455513044</t>
         </is>
       </c>
       <c r="T67" s="13" t="n">
@@ -11463,7 +11455,7 @@
       </c>
       <c r="AD67" s="13" t="inlineStr">
         <is>
-          <t>Laotian expat on a valid QID, no lines - HRN nationality coverage.</t>
+          <t>Cambodian expat on a valid QID, no lines - HRN nationality coverage.</t>
         </is>
       </c>
       <c r="AE67" s="13" t="inlineStr">
@@ -11473,7 +11465,7 @@
       </c>
       <c r="AF67" s="13" t="inlineStr">
         <is>
-          <t>HRN (Laos is on the list): QAR 100 advance and credit limit 50.</t>
+          <t>HRN (Cambodia is on the list): QAR 100 advance and credit limit 50.</t>
         </is>
       </c>
       <c r="AG67" s="13" t="inlineStr">
@@ -11495,7 +11487,7 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>CUST-3070</t>
+          <t>CUST-3069</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
@@ -11510,27 +11502,27 @@
       </c>
       <c r="E68" s="13" t="inlineStr">
         <is>
-          <t>Sipho Themba Dlamini</t>
+          <t>Khamla Somphone Vongsa</t>
         </is>
       </c>
       <c r="F68" s="13" t="inlineStr">
         <is>
-          <t>Sipho</t>
+          <t>Khamla</t>
         </is>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>Themba</t>
+          <t>Somphone</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr">
         <is>
-          <t>Dlamini</t>
+          <t>Vongsa</t>
         </is>
       </c>
       <c r="I68" s="13" t="inlineStr">
         <is>
-          <t>Swazi</t>
+          <t>Laotian</t>
         </is>
       </c>
       <c r="J68" s="13" t="inlineStr">
@@ -11545,25 +11537,25 @@
       </c>
       <c r="L68" s="13" t="inlineStr">
         <is>
-          <t>29103074800070</t>
+          <t>28910041800069</t>
         </is>
       </c>
       <c r="M68" s="13" t="inlineStr">
         <is>
-          <t>31/08/2030</t>
+          <t>31/12/2029</t>
         </is>
       </c>
       <c r="N68" s="13" t="inlineStr">
         <is>
-          <t>19/03/1991</t>
+          <t>02/10/1989</t>
         </is>
       </c>
       <c r="O68" s="13" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="P68" s="13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Q68" s="13" t="inlineStr">
@@ -11578,7 +11570,7 @@
       </c>
       <c r="S68" s="13" t="inlineStr">
         <is>
-          <t>+97455513046</t>
+          <t>+97455513045</t>
         </is>
       </c>
       <c r="T68" s="13" t="n">
@@ -11619,7 +11611,7 @@
       </c>
       <c r="AD68" s="13" t="inlineStr">
         <is>
-          <t>Swazi (Eswatini) expat on a valid QID, no lines - HRN nationality coverage.</t>
+          <t>Laotian expat on a valid QID, no lines - HRN nationality coverage.</t>
         </is>
       </c>
       <c r="AE68" s="13" t="inlineStr">
@@ -11629,7 +11621,7 @@
       </c>
       <c r="AF68" s="13" t="inlineStr">
         <is>
-          <t>HRN (Eswatini is on the list): QAR 100 advance and credit limit 50.</t>
+          <t>HRN (Laos is on the list): QAR 100 advance and credit limit 50.</t>
         </is>
       </c>
       <c r="AG68" s="13" t="inlineStr">
@@ -11651,7 +11643,7 @@
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>CUST-3071</t>
+          <t>CUST-3070</t>
         </is>
       </c>
       <c r="C69" s="14" t="inlineStr">
@@ -11661,37 +11653,37 @@
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>9 Reserved numbers</t>
+          <t>8 HRN &amp; ID classes</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
         <is>
-          <t>Khalifa Abdullah Saeed Al-Mohannadi</t>
+          <t>Sipho Themba Dlamini</t>
         </is>
       </c>
       <c r="F69" s="13" t="inlineStr">
         <is>
-          <t>Khalifa</t>
+          <t>Sipho</t>
         </is>
       </c>
       <c r="G69" s="13" t="inlineStr">
         <is>
-          <t>Abdullah Saeed</t>
+          <t>Themba</t>
         </is>
       </c>
       <c r="H69" s="13" t="inlineStr">
         <is>
-          <t>Al-Mohannadi</t>
+          <t>Dlamini</t>
         </is>
       </c>
       <c r="I69" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Swazi</t>
         </is>
       </c>
       <c r="J69" s="13" t="inlineStr">
         <is>
-          <t>Qatari</t>
+          <t>Expat (QID)</t>
         </is>
       </c>
       <c r="K69" s="13" t="inlineStr">
@@ -11701,21 +11693,21 @@
       </c>
       <c r="L69" s="13" t="inlineStr">
         <is>
-          <t>27801063400071</t>
+          <t>29103074800070</t>
         </is>
       </c>
       <c r="M69" s="13" t="inlineStr">
         <is>
-          <t>30/06/2031</t>
+          <t>31/08/2030</t>
         </is>
       </c>
       <c r="N69" s="13" t="inlineStr">
         <is>
-          <t>14/01/1978</t>
+          <t>19/03/1991</t>
         </is>
       </c>
       <c r="O69" s="13" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="P69" s="13" t="inlineStr">
         <is>
@@ -11724,24 +11716,24 @@
       </c>
       <c r="Q69" s="13" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Consumer (HRN)</t>
         </is>
       </c>
       <c r="R69" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="S69" s="13" t="inlineStr">
         <is>
-          <t>+97455513047</t>
+          <t>+97455513046</t>
         </is>
       </c>
       <c r="T69" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U69" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V69" s="13" t="n">
         <v>0</v>
@@ -11759,48 +11751,204 @@
       </c>
       <c r="Z69" s="13" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>HRN</t>
         </is>
       </c>
       <c r="AA69" s="13" t="inlineStr"/>
       <c r="AB69" s="13" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC69" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD69" s="13" t="inlineStr">
+        <is>
+          <t>Swazi (Eswatini) expat on a valid QID, no lines - HRN nationality coverage.</t>
+        </is>
+      </c>
+      <c r="AE69" s="13" t="inlineStr">
+        <is>
+          <t>New Postpaid</t>
+        </is>
+      </c>
+      <c r="AF69" s="13" t="inlineStr">
+        <is>
+          <t>HRN (Eswatini is on the list): QAR 100 advance and credit limit 50.</t>
+        </is>
+      </c>
+      <c r="AG69" s="13" t="inlineStr">
+        <is>
+          <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
+        </is>
+      </c>
+      <c r="AH69" s="13" t="inlineStr">
+        <is>
+          <t>Synthetic record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>TC-069</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>CUST-3071</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>In app - added 02/10/2026</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>9 Reserved numbers</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>Khalifa Abdullah Saeed Al-Mohannadi</t>
+        </is>
+      </c>
+      <c r="F70" s="13" t="inlineStr">
+        <is>
+          <t>Khalifa</t>
+        </is>
+      </c>
+      <c r="G70" s="13" t="inlineStr">
+        <is>
+          <t>Abdullah Saeed</t>
+        </is>
+      </c>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>Al-Mohannadi</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>Qatari</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>Qatari</t>
+        </is>
+      </c>
+      <c r="K70" s="13" t="inlineStr">
+        <is>
+          <t>QID</t>
+        </is>
+      </c>
+      <c r="L70" s="13" t="inlineStr">
+        <is>
+          <t>27801063400071</t>
+        </is>
+      </c>
+      <c r="M70" s="13" t="inlineStr">
+        <is>
+          <t>30/06/2031</t>
+        </is>
+      </c>
+      <c r="N70" s="13" t="inlineStr">
+        <is>
+          <t>14/01/1978</t>
+        </is>
+      </c>
+      <c r="O70" s="13" t="n">
+        <v>48</v>
+      </c>
+      <c r="P70" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="Q70" s="13" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="R70" s="13" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="S70" s="13" t="inlineStr">
+        <is>
+          <t>+97455513047</t>
+        </is>
+      </c>
+      <c r="T70" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="U70" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V70" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W70" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X70" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z70" s="13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="AA70" s="13" t="inlineStr"/>
+      <c r="AB70" s="13" t="inlineStr">
+        <is>
           <t>Loyalty (existing)</t>
         </is>
       </c>
-      <c r="AC69" s="13" t="inlineStr">
+      <c r="AC70" s="13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AD69" s="13" t="inlineStr">
+      <c r="AD70" s="13" t="inlineStr">
         <is>
           <t>Qatari with TWO numbers reserved for them (+97433001001 at 09:15 and +97455610140 at 14:35 on 04 Oct 2026), both held by the Retail Sales demo login.</t>
         </is>
       </c>
-      <c r="AE69" s="13" t="inlineStr">
+      <c r="AE70" s="13" t="inlineStr">
         <is>
           <t>New Postpaid (Number Selection)</t>
         </is>
       </c>
-      <c r="AF69" s="13" t="inlineStr">
+      <c r="AF70" s="13" t="inlineStr">
         <is>
           <t>Number Selection opens on the Reserved Numbers tab. Both holds show their reservation date and time, newest first, and the most recent (+97455610140, 14:35) is selected by default.</t>
         </is>
       </c>
-      <c r="AG69" s="13" t="inlineStr">
+      <c r="AG70" s="13" t="inlineStr">
         <is>
           <t>VFQ12341, VFQ12342, VFQ12344, VFQ12345, VFQ12352</t>
         </is>
       </c>
-      <c r="AH69" s="13" t="inlineStr">
+      <c r="AH70" s="13" t="inlineStr">
         <is>
           <t>Synthetic record.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH69"/>
+  <autoFilter ref="A1:AH70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11978,7 +12126,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>TC-001 (CUST-1001); TC-040 (CUST-1003); TC-031 (CUST-3028)</t>
+          <t>TC-001 (CUST-1001); TC-041 (CUST-1003); TC-031 (CUST-3028)</t>
         </is>
       </c>
     </row>
@@ -11998,7 +12146,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>TC-068 (CUST-3071)</t>
+          <t>TC-069 (CUST-3071)</t>
         </is>
       </c>
     </row>
@@ -12134,11 +12282,11 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>TC-036 (NAS-7001); TC-037 (NAS-7002); TC-038 (NAS-7003); TC-039 (NAS-7004)</t>
+          <t>TC-036 (NAS-7001); TC-037 (NAS-7002); TC-038 (NAS-7003); TC-039 (NAS-7004); TC-040 (NAS-7006)</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12326,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>TC-041 (CUST-1004 (seeded MNP-11002)); TC-033 (CUST-3031)</t>
+          <t>TC-042 (CUST-1004 (seeded MNP-11002)); TC-033 (CUST-3031)</t>
         </is>
       </c>
     </row>
@@ -12258,7 +12406,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>TC-001 (CUST-1001 (POUT-17001)); TC-022 (CUST-1002 (POUT-17002)); TC-040 (CUST-1003 (POUT-17003, FNP-12001))</t>
+          <t>TC-001 (CUST-1001 (POUT-17001)); TC-022 (CUST-1002 (POUT-17002)); TC-041 (CUST-1003 (POUT-17003, FNP-12001))</t>
         </is>
       </c>
     </row>
@@ -12278,7 +12426,7 @@
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>TC-022 (CUST-1002); TC-020 (CUST-3017); TC-058 (CUST-3061); TC-060 (CUST-3063)</t>
+          <t>TC-022 (CUST-1002); TC-020 (CUST-3017); TC-059 (CUST-3061); TC-061 (CUST-3063)</t>
         </is>
       </c>
     </row>
@@ -12298,7 +12446,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>TC-059 (CUST-3062); TC-061 (CUST-3064)</t>
+          <t>TC-060 (CUST-3062); TC-062 (CUST-3064)</t>
         </is>
       </c>
     </row>
@@ -12318,7 +12466,7 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>TC-029 (CUST-3026 (Pakistan)); TC-058 (CUST-3061 (Bangladesh)); TC-065 (CUST-3068 (Cambodia)); TC-061 (CUST-3064 (Myanmar)); TC-066 (CUST-3069 (Laos)); TC-020 (CUST-3017 (Kenya)); TC-059 (CUST-3062 (Uganda)); TC-067 (CUST-3070 (Eswatini))</t>
+          <t>TC-029 (CUST-3026 (Pakistan)); TC-059 (CUST-3061 (Bangladesh)); TC-066 (CUST-3068 (Cambodia)); TC-062 (CUST-3064 (Myanmar)); TC-067 (CUST-3069 (Laos)); TC-020 (CUST-3017 (Kenya)); TC-060 (CUST-3062 (Uganda)); TC-068 (CUST-3070 (Eswatini))</t>
         </is>
       </c>
     </row>
@@ -12338,7 +12486,7 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>TC-062 (CUST-3065); TC-063 (CUST-3066)</t>
+          <t>TC-063 (CUST-3065); TC-064 (CUST-3066)</t>
         </is>
       </c>
     </row>
@@ -12358,7 +12506,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>TC-023 (CUST-2001); TC-064 (CUST-3067)</t>
+          <t>TC-023 (CUST-2001); TC-065 (CUST-3067)</t>
         </is>
       </c>
     </row>
@@ -12398,7 +12546,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>TC-041 (CUST-1004); TC-042 (CUST-1006); TC-049 (CUST-3046); TC-046 (CUST-3043)</t>
+          <t>TC-042 (CUST-1004); TC-043 (CUST-1006); TC-050 (CUST-3046); TC-047 (CUST-3043)</t>
         </is>
       </c>
     </row>
@@ -12418,7 +12566,7 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>TC-042 (CUST-1006); TC-053 (CUST-9001); TC-044 (CUST-3041); TC-045 (CUST-3042); TC-047 (CUST-3044)</t>
+          <t>TC-043 (CUST-1006); TC-054 (CUST-9001); TC-045 (CUST-3041); TC-046 (CUST-3042); TC-048 (CUST-3044)</t>
         </is>
       </c>
     </row>
@@ -12438,7 +12586,7 @@
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>TC-050 (CUST-3072)</t>
+          <t>TC-051 (CUST-3072)</t>
         </is>
       </c>
     </row>
@@ -12458,7 +12606,7 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>TC-051 (CUST-3073)</t>
+          <t>TC-052 (CUST-3073)</t>
         </is>
       </c>
     </row>
@@ -12478,7 +12626,7 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>TC-022 (CUST-1002); TC-021 (CUST-1005); TC-043 (CUST-1007); TC-023 (CUST-2001); TC-048 (CUST-3045)</t>
+          <t>TC-022 (CUST-1002); TC-021 (CUST-1005); TC-044 (CUST-1007); TC-023 (CUST-2001); TC-049 (CUST-3045)</t>
         </is>
       </c>
     </row>
@@ -12518,7 +12666,7 @@
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>TC-054 (CUST-3051); TC-055 (CUST-3052); TC-056 (CUST-3053); TC-057 (CUST-3054)</t>
+          <t>TC-055 (CUST-3051); TC-056 (CUST-3052); TC-057 (CUST-3053); TC-058 (CUST-3054)</t>
         </is>
       </c>
     </row>
@@ -13212,7 +13360,7 @@
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>TC-042</t>
+          <t>TC-043</t>
         </is>
       </c>
       <c r="D2" s="13" t="inlineStr">
@@ -13254,7 +13402,7 @@
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>TC-044</t>
+          <t>TC-045</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
@@ -13296,7 +13444,7 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>TC-045</t>
+          <t>TC-046</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
@@ -13338,7 +13486,7 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>TC-053</t>
+          <t>TC-054</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -13380,7 +13528,7 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>TC-052</t>
+          <t>TC-053</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
@@ -13422,7 +13570,7 @@
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>TC-047</t>
+          <t>TC-048</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -13674,7 +13822,7 @@
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>TC-058</t>
+          <t>TC-059</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
@@ -13716,7 +13864,7 @@
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>TC-060</t>
+          <t>TC-061</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -13758,7 +13906,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>TC-064</t>
+          <t>TC-065</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -13800,7 +13948,7 @@
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>TC-041</t>
+          <t>TC-042</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -13842,7 +13990,7 @@
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>TC-049</t>
+          <t>TC-050</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -13884,7 +14032,7 @@
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>TC-051</t>
+          <t>TC-052</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -13926,7 +14074,7 @@
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>TC-042</t>
+          <t>TC-043</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -13968,7 +14116,7 @@
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>TC-046</t>
+          <t>TC-047</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -14304,7 +14452,7 @@
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>TC-061</t>
+          <t>TC-062</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
@@ -14472,7 +14620,7 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>TC-050</t>
+          <t>TC-051</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -14640,7 +14788,7 @@
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>TC-049</t>
+          <t>TC-050</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
@@ -14682,7 +14830,7 @@
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>TC-058</t>
+          <t>TC-059</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -14724,7 +14872,7 @@
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>TC-059</t>
+          <t>TC-060</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -14766,7 +14914,7 @@
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>TC-060</t>
+          <t>TC-061</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -14808,7 +14956,7 @@
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>TC-061</t>
+          <t>TC-062</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
@@ -14850,7 +14998,7 @@
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>TC-065</t>
+          <t>TC-066</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -14892,7 +15040,7 @@
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>TC-066</t>
+          <t>TC-067</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
@@ -14934,7 +15082,7 @@
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>TC-067</t>
+          <t>TC-068</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -14975,7 +15123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.15" customWidth="1" min="1" max="1"/>
@@ -16373,7 +16521,7 @@
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>TC-044</t>
+          <t>TC-045</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -16395,7 +16543,7 @@
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>TC-044</t>
+          <t>TC-045</t>
         </is>
       </c>
       <c r="B65" s="13" t="inlineStr">
@@ -16417,7 +16565,7 @@
     <row r="66">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>TC-045</t>
+          <t>TC-046</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -16439,7 +16587,7 @@
     <row r="67">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>TC-045</t>
+          <t>TC-046</t>
         </is>
       </c>
       <c r="B67" s="13" t="inlineStr">
@@ -16461,7 +16609,7 @@
     <row r="68">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>TC-046</t>
+          <t>TC-047</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -16483,7 +16631,7 @@
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>TC-046</t>
+          <t>TC-047</t>
         </is>
       </c>
       <c r="B69" s="13" t="inlineStr">
@@ -16505,7 +16653,7 @@
     <row r="70">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>TC-047</t>
+          <t>TC-048</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -16527,7 +16675,7 @@
     <row r="71">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>TC-047</t>
+          <t>TC-048</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
@@ -16549,7 +16697,7 @@
     <row r="72">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>TC-048</t>
+          <t>TC-049</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -16571,7 +16719,7 @@
     <row r="73">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>TC-048</t>
+          <t>TC-049</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
@@ -16593,7 +16741,7 @@
     <row r="74">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>TC-049</t>
+          <t>TC-050</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -16615,7 +16763,7 @@
     <row r="75">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>TC-049</t>
+          <t>TC-050</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr">
@@ -16637,7 +16785,7 @@
     <row r="76">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>TC-054</t>
+          <t>TC-055</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -16659,7 +16807,7 @@
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>TC-054</t>
+          <t>TC-055</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr">
@@ -16681,7 +16829,7 @@
     <row r="78">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>TC-054</t>
+          <t>TC-055</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -16703,7 +16851,7 @@
     <row r="79">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>TC-055</t>
+          <t>TC-056</t>
         </is>
       </c>
       <c r="B79" s="13" t="inlineStr">
@@ -16725,7 +16873,7 @@
     <row r="80">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>TC-055</t>
+          <t>TC-056</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
@@ -16747,7 +16895,7 @@
     <row r="81">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>TC-055</t>
+          <t>TC-056</t>
         </is>
       </c>
       <c r="B81" s="13" t="inlineStr">
@@ -16769,7 +16917,7 @@
     <row r="82">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>TC-056</t>
+          <t>TC-057</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
@@ -16791,7 +16939,7 @@
     <row r="83">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>TC-056</t>
+          <t>TC-057</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
@@ -16813,7 +16961,7 @@
     <row r="84">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>TC-057</t>
+          <t>TC-058</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
@@ -16835,7 +16983,7 @@
     <row r="85">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>TC-057</t>
+          <t>TC-058</t>
         </is>
       </c>
       <c r="B85" s="13" t="inlineStr">
@@ -16857,7 +17005,7 @@
     <row r="86">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>TC-058</t>
+          <t>TC-059</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr">
@@ -16879,7 +17027,7 @@
     <row r="87">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>TC-058</t>
+          <t>TC-059</t>
         </is>
       </c>
       <c r="B87" s="13" t="inlineStr">
@@ -16901,7 +17049,7 @@
     <row r="88">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>TC-059</t>
+          <t>TC-060</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
@@ -16923,7 +17071,7 @@
     <row r="89">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>TC-059</t>
+          <t>TC-060</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr">
@@ -16945,7 +17093,7 @@
     <row r="90">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>TC-059</t>
+          <t>TC-060</t>
         </is>
       </c>
       <c r="B90" s="13" t="inlineStr">
@@ -16967,7 +17115,7 @@
     <row r="91">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>TC-060</t>
+          <t>TC-061</t>
         </is>
       </c>
       <c r="B91" s="13" t="inlineStr">
@@ -16989,7 +17137,7 @@
     <row r="92">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>TC-060</t>
+          <t>TC-061</t>
         </is>
       </c>
       <c r="B92" s="13" t="inlineStr">
@@ -17011,7 +17159,7 @@
     <row r="93">
       <c r="A93" s="13" t="inlineStr">
         <is>
-          <t>TC-061</t>
+          <t>TC-062</t>
         </is>
       </c>
       <c r="B93" s="13" t="inlineStr">
@@ -17033,7 +17181,7 @@
     <row r="94">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>TC-061</t>
+          <t>TC-062</t>
         </is>
       </c>
       <c r="B94" s="13" t="inlineStr">
@@ -17055,7 +17203,7 @@
     <row r="95">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>TC-062</t>
+          <t>TC-063</t>
         </is>
       </c>
       <c r="B95" s="13" t="inlineStr">
@@ -17077,7 +17225,7 @@
     <row r="96">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>TC-062</t>
+          <t>TC-063</t>
         </is>
       </c>
       <c r="B96" s="13" t="inlineStr">
@@ -17099,7 +17247,7 @@
     <row r="97">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>TC-063</t>
+          <t>TC-064</t>
         </is>
       </c>
       <c r="B97" s="13" t="inlineStr">
@@ -17121,7 +17269,7 @@
     <row r="98">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>TC-063</t>
+          <t>TC-064</t>
         </is>
       </c>
       <c r="B98" s="13" t="inlineStr">
@@ -17143,7 +17291,7 @@
     <row r="99">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>TC-064</t>
+          <t>TC-065</t>
         </is>
       </c>
       <c r="B99" s="13" t="inlineStr">
@@ -17165,7 +17313,7 @@
     <row r="100">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>TC-064</t>
+          <t>TC-065</t>
         </is>
       </c>
       <c r="B100" s="13" t="inlineStr">
@@ -17187,7 +17335,7 @@
     <row r="101">
       <c r="A101" s="13" t="inlineStr">
         <is>
-          <t>TC-065</t>
+          <t>TC-066</t>
         </is>
       </c>
       <c r="B101" s="13" t="inlineStr">
@@ -17209,7 +17357,7 @@
     <row r="102">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>TC-065</t>
+          <t>TC-066</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
@@ -17231,7 +17379,7 @@
     <row r="103">
       <c r="A103" s="13" t="inlineStr">
         <is>
-          <t>TC-066</t>
+          <t>TC-067</t>
         </is>
       </c>
       <c r="B103" s="13" t="inlineStr">
@@ -17253,7 +17401,7 @@
     <row r="104">
       <c r="A104" s="13" t="inlineStr">
         <is>
-          <t>TC-066</t>
+          <t>TC-067</t>
         </is>
       </c>
       <c r="B104" s="13" t="inlineStr">
@@ -17275,7 +17423,7 @@
     <row r="105">
       <c r="A105" s="13" t="inlineStr">
         <is>
-          <t>TC-067</t>
+          <t>TC-068</t>
         </is>
       </c>
       <c r="B105" s="13" t="inlineStr">
@@ -17297,7 +17445,7 @@
     <row r="106">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>TC-067</t>
+          <t>TC-068</t>
         </is>
       </c>
       <c r="B106" s="13" t="inlineStr">
@@ -17319,7 +17467,7 @@
     <row r="107">
       <c r="A107" s="13" t="inlineStr">
         <is>
-          <t>TC-068</t>
+          <t>TC-069</t>
         </is>
       </c>
       <c r="B107" s="13" t="inlineStr">
@@ -17341,7 +17489,7 @@
     <row r="108">
       <c r="A108" s="13" t="inlineStr">
         <is>
-          <t>TC-068</t>
+          <t>TC-069</t>
         </is>
       </c>
       <c r="B108" s="13" t="inlineStr">
@@ -17363,7 +17511,7 @@
     <row r="109">
       <c r="A109" s="13" t="inlineStr">
         <is>
-          <t>TC-050</t>
+          <t>TC-051</t>
         </is>
       </c>
       <c r="B109" s="13" t="inlineStr">
@@ -17385,7 +17533,7 @@
     <row r="110">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>TC-050</t>
+          <t>TC-051</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
@@ -17407,7 +17555,7 @@
     <row r="111">
       <c r="A111" s="13" t="inlineStr">
         <is>
-          <t>TC-051</t>
+          <t>TC-052</t>
         </is>
       </c>
       <c r="B111" s="13" t="inlineStr">
@@ -17429,7 +17577,7 @@
     <row r="112">
       <c r="A112" s="13" t="inlineStr">
         <is>
-          <t>TC-051</t>
+          <t>TC-052</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
@@ -17671,7 +17819,7 @@
     <row r="123">
       <c r="A123" s="13" t="inlineStr">
         <is>
-          <t>TC-052</t>
+          <t>TC-053</t>
         </is>
       </c>
       <c r="B123" s="13" t="inlineStr">
@@ -17693,7 +17841,7 @@
     <row r="124">
       <c r="A124" s="13" t="inlineStr">
         <is>
-          <t>TC-052</t>
+          <t>TC-053</t>
         </is>
       </c>
       <c r="B124" s="13" t="inlineStr">
@@ -17844,8 +17992,30 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="13" t="inlineStr">
+        <is>
+          <t>TC-040</t>
+        </is>
+      </c>
+      <c r="B131" s="13" t="inlineStr">
+        <is>
+          <t>NAS-7006</t>
+        </is>
+      </c>
+      <c r="C131" s="13" t="inlineStr">
+        <is>
+          <t>nas-records.json</t>
+        </is>
+      </c>
+      <c r="D131" s="13" t="inlineStr">
+        <is>
+          <t>Add NAS record: documentType QID, documentNumber 29303051200106, expiryDate 2030-10-31, name 'Farhan Aslam Javed Chaudhry', dob 1993-03-05, nationality Pakistani, gender Male, email.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D130"/>
+  <autoFilter ref="A1:D131"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Number picker search modes and inventory, shared Pagination capability, Title Case UI, Address and Billing skip, discount and eligibility updates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
+++ b/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
@@ -2900,7 +2900,7 @@
       </c>
       <c r="AE12" s="13" t="inlineStr">
         <is>
-          <t>Customer Search; Customer 360; Customer Identification in any journey</t>
+          <t>Customer Search; Customer 360; Customer Verification in any journey</t>
         </is>
       </c>
       <c r="AF12" s="13" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="AE13" s="13" t="inlineStr">
         <is>
-          <t>Customer Search; Customer 360; Customer Identification in any journey</t>
+          <t>Customer Search; Customer 360; Customer Verification in any journey</t>
         </is>
       </c>
       <c r="AF13" s="13" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="AE14" s="13" t="inlineStr">
         <is>
-          <t>Customer Search; Customer 360; Customer Identification in any journey</t>
+          <t>Customer Search; Customer 360; Customer Verification in any journey</t>
         </is>
       </c>
       <c r="AF14" s="13" t="inlineStr">
@@ -4917,7 +4917,7 @@
       <c r="AA25" s="13" t="inlineStr"/>
       <c r="AB25" s="13" t="inlineStr">
         <is>
-          <t>MADA (-10%, ADO-7112) + Loyalty (-15%) - max ONE discount per order</t>
+          <t>MADA (-25%, ADO-7112) + Loyalty (-15%) - max ONE discount per order</t>
         </is>
       </c>
       <c r="AC25" s="13" t="inlineStr">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="AB29" s="13" t="inlineStr">
         <is>
-          <t>B2B2C (-10% on Red 500, ADO-7113)</t>
+          <t>B2B2C (-25% on Red 500, ADO-7113)</t>
         </is>
       </c>
       <c r="AC29" s="13" t="inlineStr">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="AB61" s="13" t="inlineStr">
         <is>
-          <t>B2B2C (-10% on Red 500)</t>
+          <t>B2B2C (-25% on Red 500)</t>
         </is>
       </c>
       <c r="AC61" s="13" t="inlineStr">
@@ -13222,7 +13222,7 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Supporting ID and proof document required. MADA -10% and Loyalty -15% both apply: only one discount per order.</t>
+          <t>Supporting ID and proof document required. MADA -25% and Loyalty -15% both apply: only one discount per order.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Postpaid journey: audit fixes, Document Upload and Empty State capabilities, tab hierarchy, add-on pricing models, Waive Off, number and discount flow changes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
+++ b/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF8EA43-E6E4-0E45-99E5-7A4276913784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5F54D8-F712-7443-A49C-B2D9621B86D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="20400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5043,7 +5043,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AH70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
@@ -5181,7 +5180,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="95" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:34" ht="95" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>48</v>
       </c>
@@ -5283,7 +5282,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>74</v>
       </c>
@@ -5385,7 +5384,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>91</v>
       </c>
@@ -5487,7 +5486,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>105</v>
       </c>
@@ -5589,7 +5588,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>121</v>
       </c>
@@ -5691,7 +5690,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>133</v>
       </c>
@@ -5793,7 +5792,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>148</v>
       </c>
@@ -5895,7 +5894,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>161</v>
       </c>
@@ -5997,7 +5996,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>176</v>
       </c>
@@ -6099,7 +6098,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>188</v>
       </c>
@@ -6201,7 +6200,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>201</v>
       </c>
@@ -6303,7 +6302,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>215</v>
       </c>
@@ -6405,7 +6404,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>226</v>
       </c>
@@ -6507,7 +6506,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>237</v>
       </c>
@@ -6609,7 +6608,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>253</v>
       </c>
@@ -6711,7 +6710,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>267</v>
       </c>
@@ -6813,7 +6812,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>280</v>
       </c>
@@ -6915,7 +6914,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>294</v>
       </c>
@@ -7017,7 +7016,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>306</v>
       </c>
@@ -7119,7 +7118,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>322</v>
       </c>
@@ -7323,7 +7322,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="23" spans="1:34" ht="76" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:34" ht="76" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>354</v>
       </c>
@@ -7427,7 +7426,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="24" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>374</v>
       </c>
@@ -7527,7 +7526,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="25" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>390</v>
       </c>
@@ -7629,7 +7628,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="26" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>403</v>
       </c>
@@ -7731,7 +7730,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="27" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
         <v>416</v>
       </c>
@@ -7833,7 +7832,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
         <v>429</v>
       </c>
@@ -7937,7 +7936,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>442</v>
       </c>
@@ -8041,7 +8040,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:34" ht="76" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:34" ht="76" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
         <v>455</v>
       </c>
@@ -8145,7 +8144,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>470</v>
       </c>
@@ -8247,7 +8246,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="32" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
         <v>484</v>
       </c>
@@ -8349,7 +8348,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>499</v>
       </c>
@@ -8451,7 +8450,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>510</v>
       </c>
@@ -8553,7 +8552,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>524</v>
       </c>
@@ -8655,7 +8654,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>538</v>
       </c>
@@ -8759,7 +8758,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>551</v>
       </c>
@@ -8857,7 +8856,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="38" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
         <v>566</v>
       </c>
@@ -8953,7 +8952,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
         <v>579</v>
       </c>
@@ -9049,7 +9048,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
         <v>591</v>
       </c>
@@ -9145,7 +9144,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
         <v>603</v>
       </c>
@@ -9241,7 +9240,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>613</v>
       </c>
@@ -9343,7 +9342,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="43" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>626</v>
       </c>
@@ -9445,7 +9444,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="44" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>641</v>
       </c>
@@ -9547,7 +9546,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="45" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>657</v>
       </c>
@@ -9649,7 +9648,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="46" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>669</v>
       </c>
@@ -9751,7 +9750,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>682</v>
       </c>
@@ -9851,7 +9850,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>693</v>
       </c>
@@ -9953,7 +9952,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
         <v>704</v>
       </c>
@@ -10055,7 +10054,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
         <v>715</v>
       </c>
@@ -10157,7 +10156,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
         <v>727</v>
       </c>
@@ -10259,7 +10258,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>739</v>
       </c>
@@ -10361,7 +10360,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
         <v>750</v>
       </c>
@@ -10463,7 +10462,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="54" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
         <v>760</v>
       </c>
@@ -10565,7 +10564,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
         <v>771</v>
       </c>
@@ -10667,7 +10666,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="56" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
         <v>782</v>
       </c>
@@ -10769,7 +10768,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
         <v>796</v>
       </c>
@@ -10871,7 +10870,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
         <v>806</v>
       </c>
@@ -10973,7 +10972,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="59" spans="1:34" ht="114" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:34" ht="114" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
         <v>817</v>
       </c>
@@ -11075,7 +11074,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:34" ht="95" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:34" ht="95" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
         <v>829</v>
       </c>
@@ -11177,7 +11176,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="61" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
         <v>844</v>
       </c>
@@ -11281,7 +11280,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:34" ht="76" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:34" ht="76" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
         <v>857</v>
       </c>
@@ -11383,7 +11382,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="63" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
         <v>871</v>
       </c>
@@ -11485,7 +11484,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
         <v>883</v>
       </c>
@@ -11587,7 +11586,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
         <v>894</v>
       </c>
@@ -11689,7 +11688,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="66" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
         <v>907</v>
       </c>
@@ -11791,7 +11790,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="67" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
         <v>918</v>
       </c>
@@ -11893,7 +11892,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="68" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
         <v>930</v>
       </c>
@@ -11995,7 +11994,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="69" spans="1:34" ht="38" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
         <v>942</v>
       </c>
@@ -12097,7 +12096,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="70" spans="1:34" ht="57" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
         <v>954</v>
       </c>
@@ -12200,13 +12199,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH70" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <filterColumn colId="10">
-      <filters>
-        <filter val="GCC ID"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AH70" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Public</oddFooter>

</xml_diff>

<commit_message>
Demo audit: new-customer eligibility at Product Selection, background page save, Back mirrors Continue, Track Ticket link, ID type in header, checkout name, cash payment label
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
+++ b/vfq-dxp-app/reference/outputs/02 Customer-Inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5F54D8-F712-7443-A49C-B2D9621B86D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92661412-9A0E-774F-BF77-D9F9B5BA8774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="20400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7118,51 +7118,51 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:34" ht="38" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:34" ht="95" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
-        <v>322</v>
+        <v>829</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>323</v>
+        <v>830</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>239</v>
+        <v>831</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>324</v>
+        <v>832</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>325</v>
+        <v>833</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>326</v>
+        <v>834</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>327</v>
+        <v>835</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>328</v>
+        <v>836</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>245</v>
+        <v>313</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>57</v>
+        <v>314</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>329</v>
+        <v>837</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>330</v>
+        <v>838</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>331</v>
+        <v>839</v>
       </c>
       <c r="O21" s="2">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>61</v>
@@ -7174,16 +7174,16 @@
         <v>114</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>333</v>
+        <v>840</v>
       </c>
       <c r="T21" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U21" s="2">
         <v>0</v>
       </c>
       <c r="V21" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W21" s="2">
         <v>0</v>
@@ -7205,19 +7205,19 @@
         <v>86</v>
       </c>
       <c r="AD21" s="2" t="s">
-        <v>335</v>
+        <v>841</v>
       </c>
       <c r="AE21" s="2" t="s">
-        <v>336</v>
+        <v>320</v>
       </c>
       <c r="AF21" s="2" t="s">
-        <v>337</v>
+        <v>842</v>
       </c>
       <c r="AG21" s="2" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="AH21" s="2" t="s">
-        <v>90</v>
+        <v>843</v>
       </c>
     </row>
     <row r="22" spans="1:34" ht="76" x14ac:dyDescent="0.2">
@@ -8040,33 +8040,33 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:34" ht="76" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>455</v>
+        <v>871</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>456</v>
+        <v>872</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>356</v>
+        <v>831</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>457</v>
+        <v>873</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>458</v>
+        <v>874</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>459</v>
+        <v>875</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>460</v>
+        <v>876</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>461</v>
+        <v>877</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>245</v>
@@ -8075,16 +8075,16 @@
         <v>57</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>462</v>
+        <v>878</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>463</v>
+        <v>879</v>
       </c>
       <c r="O30" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>61</v>
@@ -8093,16 +8093,16 @@
         <v>332</v>
       </c>
       <c r="R30" s="2" t="s">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="S30" s="2" t="s">
-        <v>464</v>
+        <v>880</v>
       </c>
       <c r="T30" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U30" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V30" s="2">
         <v>0</v>
@@ -8119,23 +8119,21 @@
       <c r="Z30" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="AA30" s="2" t="s">
-        <v>465</v>
-      </c>
+      <c r="AA30" s="2"/>
       <c r="AB30" s="2" t="s">
-        <v>466</v>
+        <v>85</v>
       </c>
       <c r="AC30" s="2" t="s">
         <v>86</v>
       </c>
       <c r="AD30" s="2" t="s">
-        <v>467</v>
+        <v>881</v>
       </c>
       <c r="AE30" s="2" t="s">
-        <v>468</v>
+        <v>265</v>
       </c>
       <c r="AF30" s="2" t="s">
-        <v>469</v>
+        <v>882</v>
       </c>
       <c r="AG30" s="2" t="s">
         <v>72</v>
@@ -8654,30 +8652,30 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:34" ht="57" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:34" ht="76" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>538</v>
+        <v>455</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>539</v>
+        <v>456</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>512</v>
+        <v>356</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>540</v>
+        <v>457</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>541</v>
+        <v>458</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>542</v>
+        <v>459</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>543</v>
+        <v>460</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>461</v>
@@ -8689,16 +8687,16 @@
         <v>57</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>544</v>
+        <v>462</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>330</v>
+        <v>112</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>545</v>
+        <v>463</v>
       </c>
       <c r="O36" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P36" s="2" t="s">
         <v>61</v>
@@ -8710,7 +8708,7 @@
         <v>114</v>
       </c>
       <c r="S36" s="2" t="s">
-        <v>546</v>
+        <v>464</v>
       </c>
       <c r="T36" s="2">
         <v>1</v>
@@ -8740,19 +8738,19 @@
         <v>466</v>
       </c>
       <c r="AC36" s="2" t="s">
-        <v>547</v>
+        <v>86</v>
       </c>
       <c r="AD36" s="2" t="s">
-        <v>548</v>
+        <v>467</v>
       </c>
       <c r="AE36" s="2" t="s">
-        <v>549</v>
+        <v>468</v>
       </c>
       <c r="AF36" s="2" t="s">
-        <v>550</v>
+        <v>469</v>
       </c>
       <c r="AG36" s="2" t="s">
-        <v>372</v>
+        <v>72</v>
       </c>
       <c r="AH36" s="2" t="s">
         <v>90</v>
@@ -10158,28 +10156,28 @@
     </row>
     <row r="51" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
-        <v>727</v>
+        <v>538</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>728</v>
+        <v>539</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>628</v>
+        <v>512</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>729</v>
+        <v>540</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>730</v>
+        <v>541</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>731</v>
+        <v>542</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>732</v>
+        <v>543</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>461</v>
@@ -10191,16 +10189,16 @@
         <v>57</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>733</v>
+        <v>544</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>434</v>
+        <v>330</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>734</v>
+        <v>545</v>
       </c>
       <c r="O51" s="2">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="P51" s="2" t="s">
         <v>61</v>
@@ -10212,7 +10210,7 @@
         <v>114</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>735</v>
+        <v>546</v>
       </c>
       <c r="T51" s="2">
         <v>1</v>
@@ -10230,29 +10228,31 @@
         <v>0</v>
       </c>
       <c r="Y51" s="2" t="s">
-        <v>636</v>
+        <v>65</v>
       </c>
       <c r="Z51" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="AA51" s="2"/>
+      <c r="AA51" s="2" t="s">
+        <v>465</v>
+      </c>
       <c r="AB51" s="2" t="s">
-        <v>211</v>
+        <v>466</v>
       </c>
       <c r="AC51" s="2" t="s">
-        <v>86</v>
+        <v>547</v>
       </c>
       <c r="AD51" s="2" t="s">
-        <v>736</v>
+        <v>548</v>
       </c>
       <c r="AE51" s="2" t="s">
-        <v>737</v>
+        <v>549</v>
       </c>
       <c r="AF51" s="2" t="s">
-        <v>738</v>
+        <v>550</v>
       </c>
       <c r="AG51" s="2" t="s">
-        <v>72</v>
+        <v>372</v>
       </c>
       <c r="AH51" s="2" t="s">
         <v>90</v>
@@ -11074,51 +11074,51 @@
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:34" ht="95" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:34" ht="57" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
-        <v>829</v>
+        <v>727</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>830</v>
+        <v>728</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>831</v>
+        <v>628</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>832</v>
+        <v>729</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>833</v>
+        <v>730</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>834</v>
+        <v>731</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>835</v>
+        <v>732</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>836</v>
+        <v>461</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>313</v>
+        <v>245</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>314</v>
+        <v>57</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>837</v>
+        <v>733</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>838</v>
+        <v>434</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>839</v>
+        <v>734</v>
       </c>
       <c r="O60" s="2">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="P60" s="2" t="s">
         <v>61</v>
@@ -11130,16 +11130,16 @@
         <v>114</v>
       </c>
       <c r="S60" s="2" t="s">
-        <v>840</v>
+        <v>735</v>
       </c>
       <c r="T60" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U60" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V60" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W60" s="2">
         <v>0</v>
@@ -11148,7 +11148,7 @@
         <v>0</v>
       </c>
       <c r="Y60" s="2" t="s">
-        <v>65</v>
+        <v>636</v>
       </c>
       <c r="Z60" s="2" t="s">
         <v>334</v>
@@ -11161,19 +11161,19 @@
         <v>86</v>
       </c>
       <c r="AD60" s="2" t="s">
-        <v>841</v>
+        <v>736</v>
       </c>
       <c r="AE60" s="2" t="s">
-        <v>320</v>
+        <v>737</v>
       </c>
       <c r="AF60" s="2" t="s">
-        <v>842</v>
+        <v>738</v>
       </c>
       <c r="AG60" s="2" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="AH60" s="2" t="s">
-        <v>843</v>
+        <v>90</v>
       </c>
     </row>
     <row r="61" spans="1:34" ht="38" x14ac:dyDescent="0.2">
@@ -11384,31 +11384,31 @@
     </row>
     <row r="63" spans="1:34" ht="38" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
-        <v>871</v>
+        <v>322</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>872</v>
+        <v>323</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>831</v>
+        <v>239</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>873</v>
+        <v>324</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>874</v>
+        <v>325</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>875</v>
+        <v>326</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>876</v>
+        <v>327</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>877</v>
+        <v>328</v>
       </c>
       <c r="J63" s="2" t="s">
         <v>245</v>
@@ -11417,16 +11417,16 @@
         <v>57</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>878</v>
+        <v>329</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>59</v>
+        <v>330</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>879</v>
+        <v>331</v>
       </c>
       <c r="O63" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P63" s="2" t="s">
         <v>61</v>
@@ -11435,16 +11435,16 @@
         <v>332</v>
       </c>
       <c r="R63" s="2" t="s">
-        <v>63</v>
+        <v>114</v>
       </c>
       <c r="S63" s="2" t="s">
-        <v>880</v>
+        <v>333</v>
       </c>
       <c r="T63" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U63" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V63" s="2">
         <v>0</v>
@@ -11463,19 +11463,19 @@
       </c>
       <c r="AA63" s="2"/>
       <c r="AB63" s="2" t="s">
-        <v>85</v>
+        <v>211</v>
       </c>
       <c r="AC63" s="2" t="s">
         <v>86</v>
       </c>
       <c r="AD63" s="2" t="s">
-        <v>881</v>
+        <v>335</v>
       </c>
       <c r="AE63" s="2" t="s">
-        <v>265</v>
+        <v>336</v>
       </c>
       <c r="AF63" s="2" t="s">
-        <v>882</v>
+        <v>337</v>
       </c>
       <c r="AG63" s="2" t="s">
         <v>72</v>

</xml_diff>